<commit_message>
Regenerate roadmap from eToro_Plus_Money_1776153611 export.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -3088,7 +3088,7 @@
         <v/>
       </c>
       <c r="F65" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V1(20.4)</v>
       </c>
       <c r="G65" t="str">
         <v/>
@@ -3123,7 +3123,7 @@
         <v/>
       </c>
       <c r="F66" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V1(20.4)</v>
       </c>
       <c r="G66" t="str">
         <v/>

</xml_diff>

<commit_message>
Regenerate roadmap from eToro_Plus_Money_1776343380 export.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -1601,7 +1601,7 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="str">
-        <v>Money Core- - Inbal</v>
+        <v>Money Core- Inbal</v>
       </c>
       <c r="B27" t="str">
         <v/>
@@ -3159,8 +3159,8 @@
       <c r="C67" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D67" s="5" t="str">
-        <v>Dev - WIP</v>
+      <c r="D67" s="11" t="str">
+        <v>Done</v>
       </c>
       <c r="E67" s="6" t="str">
         <v/>
@@ -6007,8 +6007,8 @@
       <c r="B140" t="str">
         <v/>
       </c>
-      <c r="C140" s="14" t="str">
-        <v>Discovery</v>
+      <c r="C140" s="11" t="str">
+        <v>Done</v>
       </c>
       <c r="D140" t="str">
         <v/>

</xml_diff>

<commit_message>
chore: refresh roadmap from Monday Excel export (eToro_Plus_Money_1777967429)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -64,7 +64,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -133,11 +133,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF757575"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFF5AC4"/>
       </patternFill>
     </fill>
@@ -179,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -248,9 +243,6 @@
     <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -264,7 +256,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1023,7 +1015,7 @@
         <v/>
       </c>
       <c r="F12" s="6" t="str">
-        <v>V1(20.4), V2(4.5)</v>
+        <v>V2(4.5)</v>
       </c>
       <c r="G12" t="str">
         <v/>
@@ -2498,8 +2490,8 @@
       <c r="B51" t="str">
         <v/>
       </c>
-      <c r="C51" s="19" t="str">
-        <v>Groomed</v>
+      <c r="C51" s="5" t="str">
+        <v>FE DEV WIP</v>
       </c>
       <c r="D51" t="str">
         <v/>
@@ -2776,7 +2768,7 @@
       <c r="C58" t="str">
         <v/>
       </c>
-      <c r="D58" s="20" t="str">
+      <c r="D58" s="19" t="str">
         <v>OnHold</v>
       </c>
       <c r="E58" s="6" t="str">
@@ -2811,7 +2803,7 @@
       <c r="C59" t="str">
         <v/>
       </c>
-      <c r="D59" s="21" t="str">
+      <c r="D59" s="20" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E59" s="6" t="str">
@@ -3466,7 +3458,7 @@
       <c r="C76" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D76" s="22" t="str">
+      <c r="D76" s="21" t="str">
         <v>Design</v>
       </c>
       <c r="E76" s="6" t="str">
@@ -3501,7 +3493,7 @@
       <c r="C77" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D77" s="22" t="str">
+      <c r="D77" s="21" t="str">
         <v>Design</v>
       </c>
       <c r="E77" s="6" t="str">
@@ -3846,7 +3838,7 @@
       <c r="C86" t="str">
         <v/>
       </c>
-      <c r="D86" s="21" t="str">
+      <c r="D86" s="20" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E86" s="6" t="str">
@@ -4226,7 +4218,7 @@
       <c r="C96" t="str">
         <v/>
       </c>
-      <c r="D96" s="23" t="str">
+      <c r="D96" s="22" t="str">
         <v>Grooming</v>
       </c>
       <c r="E96" s="6" t="str">
@@ -4261,7 +4253,7 @@
       <c r="C97" t="str">
         <v/>
       </c>
-      <c r="D97" s="23" t="str">
+      <c r="D97" s="22" t="str">
         <v>Grooming</v>
       </c>
       <c r="E97" s="6" t="str">
@@ -4331,7 +4323,7 @@
       <c r="C99" t="str">
         <v/>
       </c>
-      <c r="D99" s="23" t="str">
+      <c r="D99" s="22" t="str">
         <v>Grooming</v>
       </c>
       <c r="E99" s="6" t="str">
@@ -4816,7 +4808,7 @@
       <c r="C112" s="6" t="str">
         <v>Richard Whitehouse</v>
       </c>
-      <c r="D112" s="21" t="str">
+      <c r="D112" s="20" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E112" s="6" t="str">
@@ -5083,7 +5075,7 @@
       <c r="B118" t="str">
         <v/>
       </c>
-      <c r="C118" s="21" t="str">
+      <c r="C118" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D118" t="str">
@@ -5768,7 +5760,7 @@
       <c r="B135" t="str">
         <v/>
       </c>
-      <c r="C135" s="24" t="str">
+      <c r="C135" s="23" t="str">
         <v>Dependency</v>
       </c>
       <c r="D135" t="str">
@@ -5871,7 +5863,7 @@
       <c r="C137" t="str">
         <v/>
       </c>
-      <c r="D137" s="22" t="str">
+      <c r="D137" s="21" t="str">
         <v>Design</v>
       </c>
       <c r="E137" s="6" t="str">
@@ -6042,10 +6034,10 @@
       <c r="E140" t="str">
         <v/>
       </c>
-      <c r="F140" s="25">
+      <c r="F140" s="24">
         <v>46061</v>
       </c>
-      <c r="G140" s="25">
+      <c r="G140" s="24">
         <v>46160</v>
       </c>
       <c r="H140" t="str">
@@ -6063,7 +6055,7 @@
       <c r="L140" t="str">
         <v/>
       </c>
-      <c r="M140" s="26">
+      <c r="M140" s="25">
         <v>32</v>
       </c>
       <c r="N140" t="str">
@@ -6075,25 +6067,25 @@
       <c r="P140" t="str">
         <v/>
       </c>
-      <c r="Q140" s="27" t="str">
+      <c r="Q140" s="26" t="str">
         <v>2026-02-02 to 2026-04-15</v>
       </c>
       <c r="R140" t="str">
         <v/>
       </c>
-      <c r="S140" s="28" t="str">
-        <v/>
-      </c>
-      <c r="T140" s="25">
+      <c r="S140" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T140" s="24">
         <v>46058</v>
       </c>
-      <c r="U140" s="25">
+      <c r="U140" s="24">
         <v>46114</v>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="142" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" s="29" t="str">
+      <c r="A142" s="28" t="str">
         <v>In Focus</v>
       </c>
     </row>
@@ -6364,7 +6356,7 @@
       <c r="B147" t="str">
         <v/>
       </c>
-      <c r="C147" s="30" t="str">
+      <c r="C147" s="29" t="str">
         <v>Risk</v>
       </c>
       <c r="D147" t="str">
@@ -7608,10 +7600,10 @@
       <c r="E166" t="str">
         <v/>
       </c>
-      <c r="F166" s="25">
+      <c r="F166" s="24">
         <v>46054</v>
       </c>
-      <c r="G166" s="25">
+      <c r="G166" s="24">
         <v>46118</v>
       </c>
       <c r="H166" t="str">
@@ -7629,7 +7621,7 @@
       <c r="L166" t="str">
         <v/>
       </c>
-      <c r="M166" s="26">
+      <c r="M166" s="25">
         <v>0</v>
       </c>
       <c r="N166" t="str">
@@ -7641,25 +7633,25 @@
       <c r="P166" t="str">
         <v/>
       </c>
-      <c r="Q166" s="28" t="str">
+      <c r="Q166" s="27" t="str">
         <v/>
       </c>
       <c r="R166" t="str">
         <v/>
       </c>
-      <c r="S166" s="28" t="str">
-        <v/>
-      </c>
-      <c r="T166" s="28" t="str">
-        <v/>
-      </c>
-      <c r="U166" s="28" t="str">
+      <c r="S166" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T166" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U166" s="27" t="str">
         <v/>
       </c>
     </row>
     <row r="167" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="168" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" s="31" t="str">
+      <c r="A168" s="30" t="str">
         <v>MVP - API /BFF project</v>
       </c>
     </row>
@@ -9240,7 +9232,7 @@
       <c r="B201" t="str">
         <v/>
       </c>
-      <c r="C201" s="22" t="str">
+      <c r="C201" s="21" t="str">
         <v>Cancelled</v>
       </c>
       <c r="D201" s="6" t="str">
@@ -9305,7 +9297,7 @@
       <c r="B202" t="str">
         <v/>
       </c>
-      <c r="C202" s="22" t="str">
+      <c r="C202" s="21" t="str">
         <v>Cancelled</v>
       </c>
       <c r="D202" s="6" t="str">
@@ -9370,7 +9362,7 @@
       <c r="B203" t="str">
         <v/>
       </c>
-      <c r="C203" s="21" t="str">
+      <c r="C203" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D203" s="6" t="str">
@@ -9444,10 +9436,10 @@
       <c r="E204" t="str">
         <v/>
       </c>
-      <c r="F204" s="25">
+      <c r="F204" s="24">
         <v>46036</v>
       </c>
-      <c r="G204" s="25">
+      <c r="G204" s="24">
         <v>46134</v>
       </c>
       <c r="H204" t="str">
@@ -9465,7 +9457,7 @@
       <c r="L204" t="str">
         <v/>
       </c>
-      <c r="M204" s="26">
+      <c r="M204" s="25">
         <v>9</v>
       </c>
       <c r="N204" t="str">
@@ -9477,25 +9469,25 @@
       <c r="P204" t="str">
         <v/>
       </c>
-      <c r="Q204" s="28" t="str">
+      <c r="Q204" s="27" t="str">
         <v/>
       </c>
       <c r="R204" t="str">
         <v/>
       </c>
-      <c r="S204" s="28" t="str">
-        <v/>
-      </c>
-      <c r="T204" s="28" t="str">
-        <v/>
-      </c>
-      <c r="U204" s="28" t="str">
+      <c r="S204" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T204" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U204" s="27" t="str">
         <v/>
       </c>
     </row>
     <row r="205" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="206" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A206" s="32" t="str">
+      <c r="A206" s="31" t="str">
         <v>Not in Money scope/Future versions</v>
       </c>
     </row>
@@ -9571,7 +9563,7 @@
       <c r="B208" t="str">
         <v/>
       </c>
-      <c r="C208" s="21" t="str">
+      <c r="C208" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D208" s="6" t="str">
@@ -9636,7 +9628,7 @@
       <c r="B209" t="str">
         <v/>
       </c>
-      <c r="C209" s="21" t="str">
+      <c r="C209" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D209" s="6" t="str">
@@ -9701,7 +9693,7 @@
       <c r="B210" t="str">
         <v/>
       </c>
-      <c r="C210" s="21" t="str">
+      <c r="C210" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D210" s="6" t="str">
@@ -9766,7 +9758,7 @@
       <c r="B211" t="str">
         <v/>
       </c>
-      <c r="C211" s="21" t="str">
+      <c r="C211" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D211" s="6" t="str">
@@ -9831,7 +9823,7 @@
       <c r="B212" t="str">
         <v/>
       </c>
-      <c r="C212" s="21" t="str">
+      <c r="C212" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D212" s="6" t="str">
@@ -9897,7 +9889,7 @@
       <c r="B213" t="str">
         <v/>
       </c>
-      <c r="C213" s="21" t="str">
+      <c r="C213" s="20" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D213" s="6" t="str">
@@ -10067,7 +10059,7 @@
       <c r="B217" t="str">
         <v/>
       </c>
-      <c r="C217" s="20" t="str">
+      <c r="C217" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D217" s="6" t="str">
@@ -10132,7 +10124,7 @@
       <c r="B218" t="str">
         <v/>
       </c>
-      <c r="C218" s="20" t="str">
+      <c r="C218" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D218" s="6" t="str">
@@ -10197,7 +10189,7 @@
       <c r="B219" t="str">
         <v/>
       </c>
-      <c r="C219" s="20" t="str">
+      <c r="C219" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D219" t="str">
@@ -10367,7 +10359,7 @@
       <c r="B223" t="str">
         <v/>
       </c>
-      <c r="C223" s="20" t="str">
+      <c r="C223" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D223" s="6" t="str">
@@ -10432,7 +10424,7 @@
       <c r="B224" t="str">
         <v/>
       </c>
-      <c r="C224" s="20" t="str">
+      <c r="C224" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D224" s="6" t="str">
@@ -10497,7 +10489,7 @@
       <c r="B225" t="str">
         <v/>
       </c>
-      <c r="C225" s="20" t="str">
+      <c r="C225" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D225" t="str">
@@ -10562,7 +10554,7 @@
       <c r="B226" t="str">
         <v/>
       </c>
-      <c r="C226" s="20" t="str">
+      <c r="C226" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D226" t="str">
@@ -10627,7 +10619,7 @@
       <c r="B227" t="str">
         <v/>
       </c>
-      <c r="C227" s="20" t="str">
+      <c r="C227" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D227" s="6" t="str">
@@ -10692,7 +10684,7 @@
       <c r="B228" t="str">
         <v/>
       </c>
-      <c r="C228" s="22" t="str">
+      <c r="C228" s="21" t="str">
         <v>Cancelled</v>
       </c>
       <c r="D228" t="str">
@@ -10757,7 +10749,7 @@
       <c r="B229" t="str">
         <v/>
       </c>
-      <c r="C229" s="22" t="str">
+      <c r="C229" s="21" t="str">
         <v>Cancelled</v>
       </c>
       <c r="D229" s="6" t="str">
@@ -10822,7 +10814,7 @@
       <c r="B230" t="str">
         <v/>
       </c>
-      <c r="C230" s="22" t="str">
+      <c r="C230" s="21" t="str">
         <v>Cancelled</v>
       </c>
       <c r="D230" t="str">
@@ -10887,7 +10879,7 @@
       <c r="B231" t="str">
         <v/>
       </c>
-      <c r="C231" s="22" t="str">
+      <c r="C231" s="21" t="str">
         <v>Cancelled</v>
       </c>
       <c r="D231" s="6" t="str">
@@ -10952,7 +10944,7 @@
       <c r="B232" t="str">
         <v/>
       </c>
-      <c r="C232" s="20" t="str">
+      <c r="C232" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D232" t="str">
@@ -11017,7 +11009,7 @@
       <c r="B233" t="str">
         <v/>
       </c>
-      <c r="C233" s="20" t="str">
+      <c r="C233" s="19" t="str">
         <v>Future Version</v>
       </c>
       <c r="D233" s="6" t="str">
@@ -11091,10 +11083,10 @@
       <c r="E234" t="str">
         <v/>
       </c>
-      <c r="F234" s="25">
+      <c r="F234" s="24">
         <v>46061</v>
       </c>
-      <c r="G234" s="25">
+      <c r="G234" s="24">
         <v>46134</v>
       </c>
       <c r="H234" t="str">
@@ -11112,7 +11104,7 @@
       <c r="L234" t="str">
         <v/>
       </c>
-      <c r="M234" s="26">
+      <c r="M234" s="25">
         <v>1298</v>
       </c>
       <c r="N234" t="str">
@@ -11124,25 +11116,25 @@
       <c r="P234" t="str">
         <v/>
       </c>
-      <c r="Q234" s="27" t="str">
+      <c r="Q234" s="26" t="str">
         <v>2026-03-02 to 2026-03-23</v>
       </c>
       <c r="R234" t="str">
         <v/>
       </c>
-      <c r="S234" s="28" t="str">
-        <v/>
-      </c>
-      <c r="T234" s="25">
+      <c r="S234" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T234" s="24">
         <v>46104</v>
       </c>
-      <c r="U234" s="25">
+      <c r="U234" s="24">
         <v>46104</v>
       </c>
     </row>
     <row r="235" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="236" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A236" s="33" t="str">
+      <c r="A236" s="32" t="str">
         <v>Program Milestones</v>
       </c>
     </row>
@@ -11747,10 +11739,10 @@
       <c r="E246" t="str">
         <v/>
       </c>
-      <c r="F246" s="25">
+      <c r="F246" s="24">
         <v>46048</v>
       </c>
-      <c r="G246" s="25">
+      <c r="G246" s="24">
         <v>46145</v>
       </c>
       <c r="H246" t="str">
@@ -11768,7 +11760,7 @@
       <c r="L246" t="str">
         <v/>
       </c>
-      <c r="M246" s="26">
+      <c r="M246" s="25">
         <v>0</v>
       </c>
       <c r="N246" t="str">
@@ -11780,25 +11772,25 @@
       <c r="P246" t="str">
         <v/>
       </c>
-      <c r="Q246" s="28" t="str">
+      <c r="Q246" s="27" t="str">
         <v/>
       </c>
       <c r="R246" t="str">
         <v/>
       </c>
-      <c r="S246" s="28" t="str">
-        <v/>
-      </c>
-      <c r="T246" s="28" t="str">
-        <v/>
-      </c>
-      <c r="U246" s="28" t="str">
+      <c r="S246" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T246" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U246" s="27" t="str">
         <v/>
       </c>
     </row>
     <row r="247" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="248" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A248" s="29" t="str">
+      <c r="A248" s="28" t="str">
         <v>Dependencies</v>
       </c>
     </row>
@@ -11939,7 +11931,7 @@
       <c r="B251" t="str">
         <v/>
       </c>
-      <c r="C251" s="22" t="str">
+      <c r="C251" s="21" t="str">
         <v>Cancelled</v>
       </c>
       <c r="D251" t="str">
@@ -12078,10 +12070,10 @@
       <c r="E253" t="str">
         <v/>
       </c>
-      <c r="F253" s="28" t="str">
-        <v/>
-      </c>
-      <c r="G253" s="28" t="str">
+      <c r="F253" s="27" t="str">
+        <v/>
+      </c>
+      <c r="G253" s="27" t="str">
         <v/>
       </c>
       <c r="H253" t="str">
@@ -12099,7 +12091,7 @@
       <c r="L253" t="str">
         <v/>
       </c>
-      <c r="M253" s="26">
+      <c r="M253" s="25">
         <v>0</v>
       </c>
       <c r="N253" t="str">
@@ -12111,19 +12103,19 @@
       <c r="P253" t="str">
         <v/>
       </c>
-      <c r="Q253" s="28" t="str">
+      <c r="Q253" s="27" t="str">
         <v/>
       </c>
       <c r="R253" t="str">
         <v/>
       </c>
-      <c r="S253" s="28" t="str">
-        <v/>
-      </c>
-      <c r="T253" s="28" t="str">
-        <v/>
-      </c>
-      <c r="U253" s="28" t="str">
+      <c r="S253" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T253" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U253" s="27" t="str">
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh roadmap from Monday Excel export (eToro_Plus_Money_1777968129)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -93,17 +93,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00C875"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDF2F4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF9D50DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00C875"/>
       </patternFill>
     </fill>
     <fill>
@@ -793,28 +793,28 @@
         <v/>
       </c>
       <c r="B6" s="4" t="str">
-        <v>Balance Display</v>
+        <v>Export Transactions</v>
       </c>
       <c r="C6" t="str">
         <v/>
       </c>
-      <c r="D6" s="11" t="str">
-        <v>Done</v>
+      <c r="D6" s="5" t="str">
+        <v>Dev - WIP</v>
       </c>
       <c r="E6" s="6" t="str">
         <v/>
       </c>
       <c r="F6" s="6" t="str">
-        <v>V1(20.4)</v>
+        <v>V2(4.5)</v>
       </c>
       <c r="G6" t="str">
         <v/>
       </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v/>
+      <c r="H6" s="8">
+        <v>46117</v>
+      </c>
+      <c r="I6" s="8">
+        <v>46126</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -828,21 +828,21 @@
         <v/>
       </c>
       <c r="B7" s="4" t="str">
-        <v>Transactions List FE</v>
+        <v>IBAN - Add Funds to Local Account (Account Info and launch Open Banking)</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" s="11" t="str">
-        <v>Done</v>
+        <v>Stuck</v>
       </c>
       <c r="E7" s="6" t="str">
         <v/>
       </c>
       <c r="F7" s="6" t="str">
-        <v>V1(20.4)</v>
-      </c>
-      <c r="G7" t="str">
+        <v>V3(18.5)</v>
+      </c>
+      <c r="G7" s="6" t="str">
         <v/>
       </c>
       <c r="H7" t="str">
@@ -863,28 +863,28 @@
         <v/>
       </c>
       <c r="B8" s="4" t="str">
-        <v>Transactions List [BFF]- Amichai Kafka</v>
+        <v>Transactional push notifications + logic</v>
       </c>
       <c r="C8" t="str">
         <v/>
       </c>
-      <c r="D8" s="11" t="str">
-        <v>Done</v>
+      <c r="D8" s="12" t="str">
+        <v>Discovery</v>
       </c>
       <c r="E8" s="6" t="str">
         <v/>
       </c>
       <c r="F8" s="6" t="str">
-        <v>V1(20.4)</v>
+        <v>V2(4.5)</v>
       </c>
       <c r="G8" t="str">
         <v/>
       </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v/>
+      <c r="H8" s="8">
+        <v>46061</v>
+      </c>
+      <c r="I8" s="8">
+        <v>46061</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -898,12 +898,12 @@
         <v/>
       </c>
       <c r="B9" s="4" t="str">
-        <v>Account Details FE</v>
+        <v>Balance Display</v>
       </c>
       <c r="C9" t="str">
         <v/>
       </c>
-      <c r="D9" s="11" t="str">
+      <c r="D9" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E9" s="6" t="str">
@@ -915,11 +915,11 @@
       <c r="G9" t="str">
         <v/>
       </c>
-      <c r="H9" s="8">
-        <v>46064</v>
-      </c>
-      <c r="I9" s="8">
-        <v>46064</v>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -933,12 +933,12 @@
         <v/>
       </c>
       <c r="B10" s="4" t="str">
-        <v>Account Details [BFF]- Amichai Kafka</v>
+        <v>Transactions List FE</v>
       </c>
       <c r="C10" t="str">
         <v/>
       </c>
-      <c r="D10" s="11" t="str">
+      <c r="D10" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E10" s="6" t="str">
@@ -950,11 +950,11 @@
       <c r="G10" t="str">
         <v/>
       </c>
-      <c r="H10" s="8">
-        <v>46064</v>
-      </c>
-      <c r="I10" s="8">
-        <v>46064</v>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -968,12 +968,12 @@
         <v/>
       </c>
       <c r="B11" s="4" t="str">
-        <v>(Bank,Card,Internal) Transaction Types and Details</v>
+        <v>Transactions List [BFF]- Amichai Kafka</v>
       </c>
       <c r="C11" t="str">
         <v/>
       </c>
-      <c r="D11" s="11" t="str">
+      <c r="D11" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E11" s="6" t="str">
@@ -1003,28 +1003,28 @@
         <v/>
       </c>
       <c r="B12" s="4" t="str">
-        <v>Export Transactions</v>
+        <v>Account Details FE</v>
       </c>
       <c r="C12" t="str">
         <v/>
       </c>
-      <c r="D12" s="5" t="str">
-        <v>Dev - WIP</v>
+      <c r="D12" s="13" t="str">
+        <v>Done</v>
       </c>
       <c r="E12" s="6" t="str">
         <v/>
       </c>
       <c r="F12" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V1(20.4)</v>
       </c>
       <c r="G12" t="str">
         <v/>
       </c>
       <c r="H12" s="8">
-        <v>46117</v>
+        <v>46064</v>
       </c>
       <c r="I12" s="8">
-        <v>46126</v>
+        <v>46064</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1038,28 +1038,28 @@
         <v/>
       </c>
       <c r="B13" s="4" t="str">
-        <v>IBAN - Add Funds to Local Account (Account Info and launch Open Banking)</v>
+        <v>Account Details [BFF]- Amichai Kafka</v>
       </c>
       <c r="C13" t="str">
         <v/>
       </c>
-      <c r="D13" s="12" t="str">
-        <v>Stuck</v>
+      <c r="D13" s="13" t="str">
+        <v>Done</v>
       </c>
       <c r="E13" s="6" t="str">
         <v/>
       </c>
       <c r="F13" s="6" t="str">
-        <v>V3(18.5)</v>
-      </c>
-      <c r="G13" s="6" t="str">
-        <v/>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <v/>
+        <v>V1(20.4)</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" s="8">
+        <v>46064</v>
+      </c>
+      <c r="I13" s="8">
+        <v>46064</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -1073,12 +1073,12 @@
         <v/>
       </c>
       <c r="B14" s="4" t="str">
-        <v>Move Funds touchpoint</v>
+        <v>(Bank,Card,Internal) Transaction Types and Details</v>
       </c>
       <c r="C14" t="str">
         <v/>
       </c>
-      <c r="D14" s="11" t="str">
+      <c r="D14" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E14" s="6" t="str">
@@ -1090,11 +1090,11 @@
       <c r="G14" t="str">
         <v/>
       </c>
-      <c r="H14" s="8">
-        <v>46061</v>
-      </c>
-      <c r="I14" s="8">
-        <v>46061</v>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -1108,19 +1108,19 @@
         <v/>
       </c>
       <c r="B15" s="4" t="str">
-        <v>Transactional push notifications + logic</v>
+        <v>Move Funds touchpoint</v>
       </c>
       <c r="C15" t="str">
         <v/>
       </c>
       <c r="D15" s="13" t="str">
-        <v>Discovery</v>
+        <v>Done</v>
       </c>
       <c r="E15" s="6" t="str">
         <v/>
       </c>
       <c r="F15" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V1(20.4)</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -1145,7 +1145,7 @@
       <c r="B16" t="str">
         <v/>
       </c>
-      <c r="C16" s="13" t="str">
+      <c r="C16" s="12" t="str">
         <v>In QA</v>
       </c>
       <c r="D16" t="str">
@@ -1248,7 +1248,7 @@
       <c r="C18" t="str">
         <v/>
       </c>
-      <c r="D18" s="11" t="str">
+      <c r="D18" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E18" s="6" t="str">
@@ -1283,7 +1283,7 @@
       <c r="C19" t="str">
         <v/>
       </c>
-      <c r="D19" s="11" t="str">
+      <c r="D19" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E19" s="6" t="str">
@@ -1315,7 +1315,7 @@
       <c r="B20" t="str">
         <v/>
       </c>
-      <c r="C20" s="13" t="str">
+      <c r="C20" s="12" t="str">
         <v>In QA</v>
       </c>
       <c r="D20" t="str">
@@ -1418,7 +1418,7 @@
       <c r="C22" t="str">
         <v/>
       </c>
-      <c r="D22" s="11" t="str">
+      <c r="D22" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E22" s="6" t="str">
@@ -1453,7 +1453,7 @@
       <c r="C23" t="str">
         <v/>
       </c>
-      <c r="D23" s="11" t="str">
+      <c r="D23" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E23" s="6" t="str">
@@ -1488,7 +1488,7 @@
       <c r="C24" t="str">
         <v/>
       </c>
-      <c r="D24" s="11" t="str">
+      <c r="D24" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E24" s="6" t="str">
@@ -1590,7 +1590,7 @@
       <c r="B27" t="str">
         <v/>
       </c>
-      <c r="C27" s="11" t="str">
+      <c r="C27" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D27" t="str">
@@ -1933,7 +1933,7 @@
       <c r="C35" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D35" s="13" t="str">
+      <c r="D35" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E35" s="6" t="str">
@@ -1968,7 +1968,7 @@
       <c r="C36" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D36" s="13" t="str">
+      <c r="D36" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E36" s="6" t="str">
@@ -2003,7 +2003,7 @@
       <c r="C37" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D37" s="12" t="str">
+      <c r="D37" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="E37" s="6" t="str">
@@ -2038,7 +2038,7 @@
       <c r="C38" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D38" s="13" t="str">
+      <c r="D38" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E38" s="6" t="str">
@@ -2073,7 +2073,7 @@
       <c r="C39" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D39" s="13" t="str">
+      <c r="D39" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E39" s="6" t="str">
@@ -2108,7 +2108,7 @@
       <c r="C40" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D40" s="13" t="str">
+      <c r="D40" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E40" s="6" t="str">
@@ -2143,7 +2143,7 @@
       <c r="C41" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D41" s="13" t="str">
+      <c r="D41" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E41" s="6" t="str">
@@ -2178,7 +2178,7 @@
       <c r="C42" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D42" s="13" t="str">
+      <c r="D42" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E42" s="6" t="str">
@@ -2458,7 +2458,7 @@
       <c r="C50" t="str">
         <v/>
       </c>
-      <c r="D50" s="13" t="str">
+      <c r="D50" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E50" s="6" t="str">
@@ -3143,7 +3143,7 @@
       <c r="C67" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D67" s="11" t="str">
+      <c r="D67" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E67" s="6" t="str">
@@ -3178,7 +3178,7 @@
       <c r="C68" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D68" s="11" t="str">
+      <c r="D68" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E68" s="6" t="str">
@@ -3213,7 +3213,7 @@
       <c r="C69" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D69" s="11" t="str">
+      <c r="D69" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E69" s="6" t="str">
@@ -3248,7 +3248,7 @@
       <c r="C70" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D70" s="11" t="str">
+      <c r="D70" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E70" s="6" t="str">
@@ -3525,7 +3525,7 @@
       <c r="B78" t="str">
         <v/>
       </c>
-      <c r="C78" s="13" t="str">
+      <c r="C78" s="12" t="str">
         <v>In QA</v>
       </c>
       <c r="D78" s="6" t="str">
@@ -3628,7 +3628,7 @@
       <c r="C80" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D80" s="11" t="str">
+      <c r="D80" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E80" s="6" t="str">
@@ -3663,7 +3663,7 @@
       <c r="C81" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D81" s="11" t="str">
+      <c r="D81" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E81" s="6" t="str">
@@ -3698,7 +3698,7 @@
       <c r="C82" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D82" s="11" t="str">
+      <c r="D82" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E82" s="6" t="str">
@@ -3733,7 +3733,7 @@
       <c r="C83" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D83" s="11" t="str">
+      <c r="D83" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E83" s="6" t="str">
@@ -3768,7 +3768,7 @@
       <c r="C84" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D84" s="11" t="str">
+      <c r="D84" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E84" s="6" t="str">
@@ -4458,7 +4458,7 @@
       <c r="C102" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D102" s="11" t="str">
+      <c r="D102" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E102" s="6" t="str">
@@ -4598,7 +4598,7 @@
       <c r="C106" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D106" s="11" t="str">
+      <c r="D106" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E106" s="6" t="str">
@@ -4773,7 +4773,7 @@
       <c r="C111" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D111" s="13" t="str">
+      <c r="D111" s="12" t="str">
         <v>Discovery</v>
       </c>
       <c r="E111" s="6" t="str">
@@ -5345,8 +5345,8 @@
       <c r="B124" t="str">
         <v/>
       </c>
-      <c r="C124" s="16" t="str">
-        <v>Deployment</v>
+      <c r="C124" s="13" t="str">
+        <v>Done</v>
       </c>
       <c r="D124" t="str">
         <v/>
@@ -5448,7 +5448,7 @@
       <c r="C126" s="6" t="str">
         <v>Hagit Zamir</v>
       </c>
-      <c r="D126" s="11" t="str">
+      <c r="D126" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E126" s="6" t="str">
@@ -5483,7 +5483,7 @@
       <c r="C127" t="str">
         <v/>
       </c>
-      <c r="D127" s="11" t="str">
+      <c r="D127" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E127" s="6" t="str">
@@ -5518,8 +5518,8 @@
       <c r="C128" t="str">
         <v/>
       </c>
-      <c r="D128" s="13" t="str">
-        <v>Discovery</v>
+      <c r="D128" s="14" t="str">
+        <v>Handle by other team</v>
       </c>
       <c r="E128" s="6" t="str">
         <v/>
@@ -5553,8 +5553,8 @@
       <c r="C129" t="str">
         <v/>
       </c>
-      <c r="D129" s="17" t="str">
-        <v>Not Started</v>
+      <c r="D129" s="14" t="str">
+        <v>Handle by other team</v>
       </c>
       <c r="E129" s="6" t="str">
         <v/>
@@ -5588,8 +5588,8 @@
       <c r="C130" t="str">
         <v/>
       </c>
-      <c r="D130" s="17" t="str">
-        <v>Not Started</v>
+      <c r="D130" s="14" t="str">
+        <v>Handle by other team</v>
       </c>
       <c r="E130" s="6" t="str">
         <v/>
@@ -6161,7 +6161,7 @@
       <c r="B144" t="str">
         <v/>
       </c>
-      <c r="C144" s="11" t="str">
+      <c r="C144" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D144" t="str">
@@ -6421,7 +6421,7 @@
       <c r="B148" t="str">
         <v/>
       </c>
-      <c r="C148" s="11" t="str">
+      <c r="C148" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D148" t="str">
@@ -6486,7 +6486,7 @@
       <c r="B149" t="str">
         <v/>
       </c>
-      <c r="C149" s="11" t="str">
+      <c r="C149" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D149" t="str">
@@ -6551,7 +6551,7 @@
       <c r="B150" t="str">
         <v/>
       </c>
-      <c r="C150" s="11" t="str">
+      <c r="C150" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D150" t="str">
@@ -6616,7 +6616,7 @@
       <c r="B151" t="str">
         <v/>
       </c>
-      <c r="C151" s="11" t="str">
+      <c r="C151" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D151" t="str">
@@ -6681,7 +6681,7 @@
       <c r="B152" t="str">
         <v/>
       </c>
-      <c r="C152" s="11" t="str">
+      <c r="C152" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D152" t="str">
@@ -6746,7 +6746,7 @@
       <c r="B153" t="str">
         <v/>
       </c>
-      <c r="C153" s="11" t="str">
+      <c r="C153" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D153" t="str">
@@ -6811,7 +6811,7 @@
       <c r="B154" t="str">
         <v/>
       </c>
-      <c r="C154" s="11" t="str">
+      <c r="C154" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D154" t="str">
@@ -6876,7 +6876,7 @@
       <c r="B155" t="str">
         <v/>
       </c>
-      <c r="C155" s="11" t="str">
+      <c r="C155" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D155" t="str">
@@ -6941,7 +6941,7 @@
       <c r="B156" t="str">
         <v/>
       </c>
-      <c r="C156" s="11" t="str">
+      <c r="C156" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D156" t="str">
@@ -7006,7 +7006,7 @@
       <c r="B157" t="str">
         <v/>
       </c>
-      <c r="C157" s="11" t="str">
+      <c r="C157" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D157" t="str">
@@ -7071,7 +7071,7 @@
       <c r="B158" t="str">
         <v/>
       </c>
-      <c r="C158" s="11" t="str">
+      <c r="C158" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D158" s="6" t="str">
@@ -7136,7 +7136,7 @@
       <c r="B159" t="str">
         <v/>
       </c>
-      <c r="C159" s="11" t="str">
+      <c r="C159" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D159" t="str">
@@ -7201,7 +7201,7 @@
       <c r="B160" t="str">
         <v/>
       </c>
-      <c r="C160" s="11" t="str">
+      <c r="C160" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D160" t="str">
@@ -7266,7 +7266,7 @@
       <c r="B161" t="str">
         <v/>
       </c>
-      <c r="C161" s="11" t="str">
+      <c r="C161" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D161" t="str">
@@ -7331,7 +7331,7 @@
       <c r="B162" t="str">
         <v/>
       </c>
-      <c r="C162" s="11" t="str">
+      <c r="C162" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D162" t="str">
@@ -7396,7 +7396,7 @@
       <c r="B163" t="str">
         <v/>
       </c>
-      <c r="C163" s="11" t="str">
+      <c r="C163" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D163" t="str">
@@ -7461,7 +7461,7 @@
       <c r="B164" t="str">
         <v/>
       </c>
-      <c r="C164" s="11" t="str">
+      <c r="C164" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D164" t="str">
@@ -7526,7 +7526,7 @@
       <c r="B165" t="str">
         <v/>
       </c>
-      <c r="C165" s="11" t="str">
+      <c r="C165" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D165" t="str">
@@ -7727,7 +7727,7 @@
       <c r="B170" t="str">
         <v/>
       </c>
-      <c r="C170" s="11" t="str">
+      <c r="C170" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D170" s="6" t="str">
@@ -7830,7 +7830,7 @@
       <c r="C172" t="str">
         <v/>
       </c>
-      <c r="D172" s="11" t="str">
+      <c r="D172" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E172" s="6" t="str">
@@ -7865,7 +7865,7 @@
       <c r="C173" t="str">
         <v/>
       </c>
-      <c r="D173" s="11" t="str">
+      <c r="D173" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E173" s="6" t="str">
@@ -7900,7 +7900,7 @@
       <c r="C174" s="6" t="str">
         <v>Hagit Zamir</v>
       </c>
-      <c r="D174" s="11" t="str">
+      <c r="D174" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E174" s="6" t="str">
@@ -7935,7 +7935,7 @@
       <c r="C175" t="str">
         <v/>
       </c>
-      <c r="D175" s="11" t="str">
+      <c r="D175" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E175" s="6" t="str">
@@ -7970,7 +7970,7 @@
       <c r="C176" t="str">
         <v/>
       </c>
-      <c r="D176" s="11" t="str">
+      <c r="D176" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E176" s="6" t="str">
@@ -8005,7 +8005,7 @@
       <c r="C177" t="str">
         <v/>
       </c>
-      <c r="D177" s="11" t="str">
+      <c r="D177" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E177" s="6" t="str">
@@ -8040,7 +8040,7 @@
       <c r="C178" t="str">
         <v/>
       </c>
-      <c r="D178" s="11" t="str">
+      <c r="D178" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E178" s="6" t="str">
@@ -8072,7 +8072,7 @@
       <c r="B179" t="str">
         <v/>
       </c>
-      <c r="C179" s="11" t="str">
+      <c r="C179" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D179" s="6" t="str">
@@ -8137,7 +8137,7 @@
       <c r="B180" t="str">
         <v/>
       </c>
-      <c r="C180" s="11" t="str">
+      <c r="C180" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D180" s="6" t="str">
@@ -8240,7 +8240,7 @@
       <c r="C182" t="str">
         <v/>
       </c>
-      <c r="D182" s="11" t="str">
+      <c r="D182" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E182" s="6" t="str">
@@ -8275,7 +8275,7 @@
       <c r="C183" t="str">
         <v/>
       </c>
-      <c r="D183" s="11" t="str">
+      <c r="D183" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E183" s="6" t="str">
@@ -8310,7 +8310,7 @@
       <c r="C184" t="str">
         <v/>
       </c>
-      <c r="D184" s="11" t="str">
+      <c r="D184" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E184" s="6" t="str">
@@ -8345,7 +8345,7 @@
       <c r="C185" t="str">
         <v/>
       </c>
-      <c r="D185" s="11" t="str">
+      <c r="D185" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E185" s="6" t="str">
@@ -8380,7 +8380,7 @@
       <c r="C186" t="str">
         <v/>
       </c>
-      <c r="D186" s="11" t="str">
+      <c r="D186" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E186" s="6" t="str">
@@ -8415,7 +8415,7 @@
       <c r="C187" t="str">
         <v/>
       </c>
-      <c r="D187" s="11" t="str">
+      <c r="D187" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="E187" s="6" t="str">
@@ -8447,7 +8447,7 @@
       <c r="B188" t="str">
         <v/>
       </c>
-      <c r="C188" s="11" t="str">
+      <c r="C188" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D188" t="str">
@@ -8577,7 +8577,7 @@
       <c r="B190" t="str">
         <v/>
       </c>
-      <c r="C190" s="11" t="str">
+      <c r="C190" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D190" t="str">
@@ -8707,7 +8707,7 @@
       <c r="B192" t="str">
         <v/>
       </c>
-      <c r="C192" s="12" t="str">
+      <c r="C192" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="D192" s="6" t="str">
@@ -8810,7 +8810,7 @@
       <c r="C194" t="str">
         <v/>
       </c>
-      <c r="D194" s="12" t="str">
+      <c r="D194" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="E194" s="6" t="str">
@@ -8842,7 +8842,7 @@
       <c r="B195" t="str">
         <v/>
       </c>
-      <c r="C195" s="12" t="str">
+      <c r="C195" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="D195" s="6" t="str">
@@ -8907,7 +8907,7 @@
       <c r="B196" t="str">
         <v/>
       </c>
-      <c r="C196" s="12" t="str">
+      <c r="C196" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="D196" s="6" t="str">
@@ -11210,7 +11210,7 @@
       <c r="B238" t="str">
         <v/>
       </c>
-      <c r="C238" s="11" t="str">
+      <c r="C238" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D238" t="str">
@@ -11866,7 +11866,7 @@
       <c r="B250" t="str">
         <v/>
       </c>
-      <c r="C250" s="11" t="str">
+      <c r="C250" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D250" t="str">
@@ -11996,7 +11996,7 @@
       <c r="B252" t="str">
         <v/>
       </c>
-      <c r="C252" s="11" t="str">
+      <c r="C252" s="13" t="str">
         <v>Done</v>
       </c>
       <c r="D252" t="str">

</xml_diff>

<commit_message>
chore: refresh roadmap from Monday Excel export (eToro_Plus_Money_1778400998)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -797,7 +797,7 @@
         <v/>
       </c>
       <c r="F6" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G6" t="str">
         <v/>
@@ -832,7 +832,7 @@
         <v/>
       </c>
       <c r="F7" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G7" s="6" t="str">
         <v/>
@@ -867,7 +867,7 @@
         <v/>
       </c>
       <c r="F8" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="F30" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G30" t="str">
         <v/>
@@ -1792,7 +1792,7 @@
         <v/>
       </c>
       <c r="F31" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G31" t="str">
         <v/>
@@ -1827,7 +1827,7 @@
         <v/>
       </c>
       <c r="F32" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G32" t="str">
         <v/>
@@ -1862,7 +1862,7 @@
         <v/>
       </c>
       <c r="F33" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G33" t="str">
         <v/>
@@ -1897,7 +1897,7 @@
         <v/>
       </c>
       <c r="F34" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G34" t="str">
         <v/>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="F35" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G35" t="str">
         <v/>
@@ -1967,7 +1967,7 @@
         <v/>
       </c>
       <c r="F36" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G36" t="str">
         <v/>
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="F37" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G37" t="str">
         <v/>
@@ -2037,7 +2037,7 @@
         <v/>
       </c>
       <c r="F38" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G38" t="str">
         <v/>
@@ -2072,7 +2072,7 @@
         <v/>
       </c>
       <c r="F39" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -2107,7 +2107,7 @@
         <v/>
       </c>
       <c r="F40" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G40" t="str">
         <v/>
@@ -2142,7 +2142,7 @@
         <v/>
       </c>
       <c r="F41" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G41" t="str">
         <v/>
@@ -2177,7 +2177,7 @@
         <v/>
       </c>
       <c r="F42" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G42" t="str">
         <v/>
@@ -2212,7 +2212,7 @@
         <v/>
       </c>
       <c r="F43" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G43" t="str">
         <v/>
@@ -2247,7 +2247,7 @@
         <v/>
       </c>
       <c r="F44" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G44" t="str">
         <v/>
@@ -2282,7 +2282,7 @@
         <v/>
       </c>
       <c r="F45" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G45" t="str">
         <v/>
@@ -2317,7 +2317,7 @@
         <v/>
       </c>
       <c r="F46" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G46" t="str">
         <v/>
@@ -3247,7 +3247,7 @@
         <v/>
       </c>
       <c r="F70" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -3282,7 +3282,7 @@
         <v/>
       </c>
       <c r="F71" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G71" t="str">
         <v/>
@@ -3317,7 +3317,7 @@
         <v/>
       </c>
       <c r="F72" s="6" t="str">
-        <v>V2(4.5)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G72" t="str">
         <v/>
@@ -3352,7 +3352,7 @@
         <v/>
       </c>
       <c r="F73" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G73" t="str">
         <v/>
@@ -3387,7 +3387,7 @@
         <v/>
       </c>
       <c r="F74" s="6" t="str">
-        <v>V3(18.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="G74" t="str">
         <v/>
@@ -3422,7 +3422,7 @@
         <v/>
       </c>
       <c r="F75" s="6" t="str">
-        <v>V4(1.6)</v>
+        <v>V4(8.6)</v>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -3457,7 +3457,7 @@
         <v/>
       </c>
       <c r="F76" s="6" t="str">
-        <v>V4(1.6)</v>
+        <v>V4(8.6)</v>
       </c>
       <c r="G76" t="str">
         <v/>

</xml_diff>

<commit_message>
chore: refresh roadmap from Monday Excel export (eToro_Plus_Money_1778402645)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -10922,7 +10922,7 @@
         <v>46134</v>
       </c>
       <c r="H232" s="6" t="str">
-        <v>V1(20.4)</v>
+        <v/>
       </c>
       <c r="I232" t="str">
         <v/>
@@ -11117,7 +11117,7 @@
         <v/>
       </c>
       <c r="H235" s="6" t="str">
-        <v>V4(8.6)</v>
+        <v/>
       </c>
       <c r="I235" t="str">
         <v/>

</xml_diff>

<commit_message>
chore: refresh roadmap from Monday Excel export (eToro_Plus_Money_1778416312)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -83,7 +83,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFDAB3D"/>
+        <fgColor rgb="FF9D50DD"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,17 +93,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00C875"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDF2F4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9D50DD"/>
+        <fgColor rgb="FF00C875"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,12 +108,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF007F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDAB3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFCAB641"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF007F"/>
+        <fgColor rgb="FF333333"/>
       </patternFill>
     </fill>
     <fill>
@@ -138,22 +143,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF333333"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFBB3354"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF66CCFF"/>
+        <fgColor rgb="FFFF5AC4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF5AC4"/>
+        <fgColor rgb="FF66CCFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -232,6 +232,9 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -245,7 +248,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -253,9 +256,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -688,7 +688,7 @@
         <v/>
       </c>
       <c r="C4" s="5" t="str">
-        <v>FE DEV WIP</v>
+        <v>In QA</v>
       </c>
       <c r="D4" s="6" t="str">
         <v>localAcctHome</v>
@@ -785,28 +785,28 @@
         <v/>
       </c>
       <c r="B6" s="4" t="str">
-        <v>Export Transactions</v>
+        <v>IBAN - Add Funds to Local Account (Account Info and launch Open Banking)</v>
       </c>
       <c r="C6" t="str">
         <v/>
       </c>
       <c r="D6" s="11" t="str">
-        <v>Done</v>
+        <v>Stuck</v>
       </c>
       <c r="E6" s="6" t="str">
         <v/>
       </c>
       <c r="F6" s="6" t="str">
-        <v>V2(11.5)</v>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" s="8">
-        <v>46117</v>
-      </c>
-      <c r="I6" s="8">
-        <v>46126</v>
+        <v>V3(25.5)</v>
+      </c>
+      <c r="G6" s="6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -820,13 +820,13 @@
         <v/>
       </c>
       <c r="B7" s="4" t="str">
-        <v>IBAN - Add Funds to Local Account (Account Info and launch Open Banking)</v>
+        <v>Transactional push notifications + logic</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
-      <c r="D7" s="12" t="str">
-        <v>Stuck</v>
+      <c r="D7" s="5" t="str">
+        <v>Discovery</v>
       </c>
       <c r="E7" s="6" t="str">
         <v/>
@@ -834,14 +834,14 @@
       <c r="F7" s="6" t="str">
         <v>V3(25.5)</v>
       </c>
-      <c r="G7" s="6" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="8">
+        <v>46061</v>
+      </c>
+      <c r="I7" s="8">
+        <v>46061</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -855,28 +855,28 @@
         <v/>
       </c>
       <c r="B8" s="4" t="str">
-        <v>Transactional push notifications + logic</v>
+        <v>Balance Display</v>
       </c>
       <c r="C8" t="str">
         <v/>
       </c>
-      <c r="D8" s="13" t="str">
-        <v>Discovery</v>
+      <c r="D8" s="12" t="str">
+        <v>Done</v>
       </c>
       <c r="E8" s="6" t="str">
         <v/>
       </c>
       <c r="F8" s="6" t="str">
-        <v>V2(11.5)</v>
+        <v>V1(20.4)</v>
       </c>
       <c r="G8" t="str">
         <v/>
       </c>
-      <c r="H8" s="8">
-        <v>46061</v>
-      </c>
-      <c r="I8" s="8">
-        <v>46061</v>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -890,12 +890,12 @@
         <v/>
       </c>
       <c r="B9" s="4" t="str">
-        <v>Balance Display</v>
+        <v>Transactions List FE</v>
       </c>
       <c r="C9" t="str">
         <v/>
       </c>
-      <c r="D9" s="11" t="str">
+      <c r="D9" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E9" s="6" t="str">
@@ -925,28 +925,28 @@
         <v/>
       </c>
       <c r="B10" s="4" t="str">
-        <v>Transactions List FE</v>
+        <v>Export Transactions</v>
       </c>
       <c r="C10" t="str">
         <v/>
       </c>
-      <c r="D10" s="11" t="str">
+      <c r="D10" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E10" s="6" t="str">
         <v/>
       </c>
       <c r="F10" s="6" t="str">
-        <v>V1(20.4)</v>
+        <v>V2(11.5)</v>
       </c>
       <c r="G10" t="str">
         <v/>
       </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v/>
+      <c r="H10" s="8">
+        <v>46117</v>
+      </c>
+      <c r="I10" s="8">
+        <v>46126</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -965,7 +965,7 @@
       <c r="C11" t="str">
         <v/>
       </c>
-      <c r="D11" s="11" t="str">
+      <c r="D11" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E11" s="6" t="str">
@@ -1000,7 +1000,7 @@
       <c r="C12" t="str">
         <v/>
       </c>
-      <c r="D12" s="11" t="str">
+      <c r="D12" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E12" s="6" t="str">
@@ -1035,7 +1035,7 @@
       <c r="C13" t="str">
         <v/>
       </c>
-      <c r="D13" s="11" t="str">
+      <c r="D13" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E13" s="6" t="str">
@@ -1070,7 +1070,7 @@
       <c r="C14" t="str">
         <v/>
       </c>
-      <c r="D14" s="11" t="str">
+      <c r="D14" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E14" s="6" t="str">
@@ -1105,7 +1105,7 @@
       <c r="C15" t="str">
         <v/>
       </c>
-      <c r="D15" s="11" t="str">
+      <c r="D15" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E15" s="6" t="str">
@@ -1137,7 +1137,7 @@
       <c r="B16" t="str">
         <v/>
       </c>
-      <c r="C16" s="13" t="str">
+      <c r="C16" s="5" t="str">
         <v>In QA</v>
       </c>
       <c r="D16" t="str">
@@ -1240,7 +1240,7 @@
       <c r="C18" t="str">
         <v/>
       </c>
-      <c r="D18" s="11" t="str">
+      <c r="D18" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E18" s="6" t="str">
@@ -1275,7 +1275,7 @@
       <c r="C19" t="str">
         <v/>
       </c>
-      <c r="D19" s="11" t="str">
+      <c r="D19" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E19" s="6" t="str">
@@ -1307,7 +1307,7 @@
       <c r="B20" t="str">
         <v/>
       </c>
-      <c r="C20" s="13" t="str">
+      <c r="C20" s="5" t="str">
         <v>In QA</v>
       </c>
       <c r="D20" t="str">
@@ -1410,7 +1410,7 @@
       <c r="C22" t="str">
         <v/>
       </c>
-      <c r="D22" s="11" t="str">
+      <c r="D22" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E22" s="6" t="str">
@@ -1445,7 +1445,7 @@
       <c r="C23" t="str">
         <v/>
       </c>
-      <c r="D23" s="11" t="str">
+      <c r="D23" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E23" s="6" t="str">
@@ -1480,7 +1480,7 @@
       <c r="C24" t="str">
         <v/>
       </c>
-      <c r="D24" s="11" t="str">
+      <c r="D24" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E24" s="6" t="str">
@@ -1510,12 +1510,12 @@
         <v/>
       </c>
       <c r="B25" s="4" t="str">
-        <v>Portfolio touchpoints - move funds- Roy- Ilan to check status</v>
+        <v>Portfolio touchpoints - move funds- Roy-Inbal  to check status</v>
       </c>
       <c r="C25" t="str">
         <v/>
       </c>
-      <c r="D25" s="14" t="str">
+      <c r="D25" s="13" t="str">
         <v>Handle by other team</v>
       </c>
       <c r="E25" s="6" t="str">
@@ -1545,19 +1545,19 @@
         <v/>
       </c>
       <c r="B26" s="4" t="str">
-        <v>Execution pop-up  Open &amp; close - move funds- Roy- Ilan to check status</v>
+        <v>Execution pop-up  Open &amp; close - move funds-</v>
       </c>
       <c r="C26" t="str">
         <v/>
       </c>
-      <c r="D26" s="12" t="str">
-        <v>Stuck</v>
+      <c r="D26" s="14" t="str">
+        <v>Groomed</v>
       </c>
       <c r="E26" s="6" t="str">
         <v/>
       </c>
-      <c r="F26" t="str">
-        <v/>
+      <c r="F26" s="6" t="str">
+        <v>V3(25.5)</v>
       </c>
       <c r="G26" t="str">
         <v/>
@@ -1582,7 +1582,7 @@
       <c r="B27" t="str">
         <v/>
       </c>
-      <c r="C27" s="11" t="str">
+      <c r="C27" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D27" t="str">
@@ -1647,7 +1647,7 @@
       <c r="B28" t="str">
         <v/>
       </c>
-      <c r="C28" s="5" t="str">
+      <c r="C28" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D28" s="6" t="str">
@@ -1750,7 +1750,7 @@
       <c r="C30" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D30" s="15" t="str">
+      <c r="D30" s="16" t="str">
         <v>QA</v>
       </c>
       <c r="E30" s="6" t="str">
@@ -1785,7 +1785,7 @@
       <c r="C31" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D31" s="15" t="str">
+      <c r="D31" s="16" t="str">
         <v>QA</v>
       </c>
       <c r="E31" s="6" t="str">
@@ -1820,7 +1820,7 @@
       <c r="C32" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D32" s="16" t="str">
+      <c r="D32" s="14" t="str">
         <v>Groomed</v>
       </c>
       <c r="E32" s="6" t="str">
@@ -1855,8 +1855,8 @@
       <c r="C33" s="6" t="str">
         <v>Noit Hoffman, Joanna Fajga</v>
       </c>
-      <c r="D33" s="16" t="str">
-        <v>Groomed</v>
+      <c r="D33" s="15" t="str">
+        <v>Dev - WIP</v>
       </c>
       <c r="E33" s="6" t="str">
         <v/>
@@ -1890,7 +1890,7 @@
       <c r="C34" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D34" s="15" t="str">
+      <c r="D34" s="16" t="str">
         <v>QA</v>
       </c>
       <c r="E34" s="6" t="str">
@@ -1925,8 +1925,8 @@
       <c r="C35" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D35" s="13" t="str">
-        <v>Discovery</v>
+      <c r="D35" s="17" t="str">
+        <v>Grooming</v>
       </c>
       <c r="E35" s="6" t="str">
         <v/>
@@ -1960,7 +1960,7 @@
       <c r="C36" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D36" s="13" t="str">
+      <c r="D36" s="5" t="str">
         <v>Discovery</v>
       </c>
       <c r="E36" s="6" t="str">
@@ -1995,7 +1995,7 @@
       <c r="C37" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D37" s="17" t="str">
+      <c r="D37" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E37" s="6" t="str">
@@ -2030,7 +2030,7 @@
       <c r="C38" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D38" s="17" t="str">
+      <c r="D38" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E38" s="6" t="str">
@@ -2065,7 +2065,7 @@
       <c r="C39" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D39" s="17" t="str">
+      <c r="D39" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E39" s="6" t="str">
@@ -2100,7 +2100,7 @@
       <c r="C40" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D40" s="17" t="str">
+      <c r="D40" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E40" s="6" t="str">
@@ -2135,7 +2135,7 @@
       <c r="C41" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D41" s="17" t="str">
+      <c r="D41" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E41" s="6" t="str">
@@ -2170,7 +2170,7 @@
       <c r="C42" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D42" s="17" t="str">
+      <c r="D42" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E42" s="6" t="str">
@@ -2205,7 +2205,7 @@
       <c r="C43" t="str">
         <v/>
       </c>
-      <c r="D43" s="5" t="str">
+      <c r="D43" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E43" s="6" t="str">
@@ -2240,7 +2240,7 @@
       <c r="C44" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D44" s="16" t="str">
+      <c r="D44" s="14" t="str">
         <v>Groomed</v>
       </c>
       <c r="E44" s="6" t="str">
@@ -2275,7 +2275,7 @@
       <c r="C45" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D45" s="16" t="str">
+      <c r="D45" s="14" t="str">
         <v>Groomed</v>
       </c>
       <c r="E45" s="6" t="str">
@@ -2310,7 +2310,7 @@
       <c r="C46" t="str">
         <v/>
       </c>
-      <c r="D46" s="18" t="str">
+      <c r="D46" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="E46" s="6" t="str">
@@ -2345,7 +2345,7 @@
       <c r="C47" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D47" s="19" t="str">
+      <c r="D47" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E47" s="6" t="str">
@@ -2380,7 +2380,7 @@
       <c r="C48" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D48" s="19" t="str">
+      <c r="D48" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E48" s="6" t="str">
@@ -2415,7 +2415,7 @@
       <c r="C49" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D49" s="19" t="str">
+      <c r="D49" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E49" s="6" t="str">
@@ -2450,14 +2450,14 @@
       <c r="C50" t="str">
         <v/>
       </c>
-      <c r="D50" s="13" t="str">
+      <c r="D50" s="5" t="str">
         <v>Discovery</v>
       </c>
       <c r="E50" s="6" t="str">
         <v/>
       </c>
-      <c r="F50" t="str">
-        <v/>
+      <c r="F50" s="6" t="str">
+        <v>V3(25.5)</v>
       </c>
       <c r="G50" t="str">
         <v/>
@@ -2482,7 +2482,7 @@
       <c r="B51" t="str">
         <v/>
       </c>
-      <c r="C51" s="5" t="str">
+      <c r="C51" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D51" t="str">
@@ -2585,7 +2585,7 @@
       <c r="C53" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D53" s="5" t="str">
+      <c r="D53" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E53" s="6" t="str">
@@ -2620,7 +2620,7 @@
       <c r="C54" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D54" s="5" t="str">
+      <c r="D54" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E54" s="6" t="str">
@@ -2655,7 +2655,7 @@
       <c r="C55" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D55" s="5" t="str">
+      <c r="D55" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E55" s="6" t="str">
@@ -2690,7 +2690,7 @@
       <c r="C56" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D56" s="5" t="str">
+      <c r="D56" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E56" s="6" t="str">
@@ -2725,7 +2725,7 @@
       <c r="C57" s="6" t="str">
         <v>Noit Hoffman</v>
       </c>
-      <c r="D57" s="5" t="str">
+      <c r="D57" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E57" s="6" t="str">
@@ -2760,7 +2760,7 @@
       <c r="C58" t="str">
         <v/>
       </c>
-      <c r="D58" s="11" t="str">
+      <c r="D58" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E58" s="6" t="str">
@@ -2795,7 +2795,7 @@
       <c r="C59" t="str">
         <v/>
       </c>
-      <c r="D59" s="17" t="str">
+      <c r="D59" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E59" s="6" t="str">
@@ -2830,7 +2830,7 @@
       <c r="C60" t="str">
         <v/>
       </c>
-      <c r="D60" s="5" t="str">
+      <c r="D60" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E60" s="6" t="str">
@@ -2862,7 +2862,7 @@
       <c r="B61" t="str">
         <v/>
       </c>
-      <c r="C61" s="15" t="str">
+      <c r="C61" s="16" t="str">
         <v>Grooming</v>
       </c>
       <c r="D61" s="6" t="str">
@@ -2878,7 +2878,7 @@
         <v/>
       </c>
       <c r="H61" s="6" t="str">
-        <v>V3(25.5)</v>
+        <v>V4(8.6)</v>
       </c>
       <c r="I61" t="str">
         <v/>
@@ -2965,7 +2965,7 @@
       <c r="C63" t="str">
         <v/>
       </c>
-      <c r="D63" s="20" t="str">
+      <c r="D63" s="17" t="str">
         <v>Grooming</v>
       </c>
       <c r="E63" s="6" t="str">
@@ -3000,7 +3000,7 @@
       <c r="C64" t="str">
         <v/>
       </c>
-      <c r="D64" s="20" t="str">
+      <c r="D64" s="17" t="str">
         <v>Grooming</v>
       </c>
       <c r="E64" s="6" t="str">
@@ -3035,7 +3035,7 @@
       <c r="C65" t="str">
         <v/>
       </c>
-      <c r="D65" s="20" t="str">
+      <c r="D65" s="17" t="str">
         <v>Grooming</v>
       </c>
       <c r="E65" s="6" t="str">
@@ -3067,7 +3067,7 @@
       <c r="B66" t="str">
         <v/>
       </c>
-      <c r="C66" s="5" t="str">
+      <c r="C66" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D66" s="6" t="str">
@@ -3170,7 +3170,7 @@
       <c r="C68" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D68" s="11" t="str">
+      <c r="D68" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E68" s="6" t="str">
@@ -3205,7 +3205,7 @@
       <c r="C69" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D69" s="11" t="str">
+      <c r="D69" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E69" s="6" t="str">
@@ -3240,7 +3240,7 @@
       <c r="C70" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D70" s="11" t="str">
+      <c r="D70" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E70" s="6" t="str">
@@ -3275,7 +3275,7 @@
       <c r="C71" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D71" s="11" t="str">
+      <c r="D71" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E71" s="6" t="str">
@@ -3310,7 +3310,7 @@
       <c r="C72" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D72" s="11" t="str">
+      <c r="D72" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E72" s="6" t="str">
@@ -3345,8 +3345,8 @@
       <c r="C73" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D73" s="16" t="str">
-        <v>Groomed</v>
+      <c r="D73" s="15" t="str">
+        <v>Dev - WIP</v>
       </c>
       <c r="E73" s="6" t="str">
         <v/>
@@ -3380,7 +3380,7 @@
       <c r="C74" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D74" s="16" t="str">
+      <c r="D74" s="14" t="str">
         <v>Groomed</v>
       </c>
       <c r="E74" s="6" t="str">
@@ -3415,7 +3415,7 @@
       <c r="C75" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D75" s="16" t="str">
+      <c r="D75" s="14" t="str">
         <v>Groomed</v>
       </c>
       <c r="E75" s="6" t="str">
@@ -3450,7 +3450,7 @@
       <c r="C76" s="6" t="str">
         <v>Nikolaus Kulier</v>
       </c>
-      <c r="D76" s="16" t="str">
+      <c r="D76" s="14" t="str">
         <v>Groomed</v>
       </c>
       <c r="E76" s="6" t="str">
@@ -3552,7 +3552,7 @@
       <c r="B79" t="str">
         <v/>
       </c>
-      <c r="C79" s="13" t="str">
+      <c r="C79" s="5" t="str">
         <v>In QA</v>
       </c>
       <c r="D79" s="6" t="str">
@@ -3655,7 +3655,7 @@
       <c r="C81" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D81" s="11" t="str">
+      <c r="D81" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E81" s="6" t="str">
@@ -3690,7 +3690,7 @@
       <c r="C82" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D82" s="11" t="str">
+      <c r="D82" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E82" s="6" t="str">
@@ -3725,7 +3725,7 @@
       <c r="C83" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D83" s="11" t="str">
+      <c r="D83" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E83" s="6" t="str">
@@ -3760,7 +3760,7 @@
       <c r="C84" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D84" s="11" t="str">
+      <c r="D84" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E84" s="6" t="str">
@@ -3795,7 +3795,7 @@
       <c r="C85" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D85" s="11" t="str">
+      <c r="D85" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E85" s="6" t="str">
@@ -3830,7 +3830,7 @@
       <c r="C86" t="str">
         <v/>
       </c>
-      <c r="D86" s="18" t="str">
+      <c r="D86" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="E86" s="6" t="str">
@@ -3865,7 +3865,7 @@
       <c r="C87" t="str">
         <v/>
       </c>
-      <c r="D87" s="17" t="str">
+      <c r="D87" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E87" s="6" t="str">
@@ -3900,7 +3900,7 @@
       <c r="C88" t="str">
         <v/>
       </c>
-      <c r="D88" s="19" t="str">
+      <c r="D88" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E88" s="6" t="str">
@@ -3935,7 +3935,7 @@
       <c r="C89" t="str">
         <v/>
       </c>
-      <c r="D89" s="19" t="str">
+      <c r="D89" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E89" s="6" t="str">
@@ -3970,7 +3970,7 @@
       <c r="C90" t="str">
         <v/>
       </c>
-      <c r="D90" s="19" t="str">
+      <c r="D90" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E90" s="6" t="str">
@@ -4005,7 +4005,7 @@
       <c r="C91" t="str">
         <v/>
       </c>
-      <c r="D91" s="19" t="str">
+      <c r="D91" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E91" s="6" t="str">
@@ -4040,7 +4040,7 @@
       <c r="C92" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D92" s="19" t="str">
+      <c r="D92" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E92" s="6" t="str">
@@ -4075,7 +4075,7 @@
       <c r="C93" t="str">
         <v/>
       </c>
-      <c r="D93" s="14" t="str">
+      <c r="D93" s="13" t="str">
         <v>Handle by other team</v>
       </c>
       <c r="E93" s="6" t="str">
@@ -4110,7 +4110,7 @@
       <c r="C94" s="6" t="str">
         <v>Joanna Fajga</v>
       </c>
-      <c r="D94" s="19" t="str">
+      <c r="D94" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E94" s="6" t="str">
@@ -4142,7 +4142,7 @@
       <c r="B95" t="str">
         <v/>
       </c>
-      <c r="C95" s="15" t="str">
+      <c r="C95" s="16" t="str">
         <v>Grooming</v>
       </c>
       <c r="D95" s="6" t="str">
@@ -4158,7 +4158,7 @@
         <v>46134</v>
       </c>
       <c r="H95" s="6" t="str">
-        <v>V3(25.5)</v>
+        <v>V4(8.6)</v>
       </c>
       <c r="I95" s="6" t="str">
         <v>BFF</v>
@@ -4245,7 +4245,7 @@
       <c r="C97" t="str">
         <v/>
       </c>
-      <c r="D97" s="20" t="str">
+      <c r="D97" s="17" t="str">
         <v>Grooming</v>
       </c>
       <c r="E97" s="6" t="str">
@@ -4280,7 +4280,7 @@
       <c r="C98" t="str">
         <v/>
       </c>
-      <c r="D98" s="20" t="str">
+      <c r="D98" s="17" t="str">
         <v>Grooming</v>
       </c>
       <c r="E98" s="6" t="str">
@@ -4315,7 +4315,7 @@
       <c r="C99" t="str">
         <v/>
       </c>
-      <c r="D99" s="18" t="str">
+      <c r="D99" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="E99" s="6" t="str">
@@ -4350,7 +4350,7 @@
       <c r="C100" t="str">
         <v/>
       </c>
-      <c r="D100" s="20" t="str">
+      <c r="D100" s="17" t="str">
         <v>Grooming</v>
       </c>
       <c r="E100" s="6" t="str">
@@ -4382,7 +4382,7 @@
       <c r="B101" t="str">
         <v/>
       </c>
-      <c r="C101" s="5" t="str">
+      <c r="C101" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D101" s="6" t="str">
@@ -4398,7 +4398,7 @@
         <v>46154</v>
       </c>
       <c r="H101" s="6" t="str">
-        <v>V2(11.5)</v>
+        <v>V3(25.5)</v>
       </c>
       <c r="I101" s="6" t="str">
         <v>Freeze Card and Card Status mgmt still requires Design</v>
@@ -4485,7 +4485,7 @@
       <c r="C103" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D103" s="11" t="str">
+      <c r="D103" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E103" s="6" t="str">
@@ -4520,8 +4520,8 @@
       <c r="C104" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D104" s="16" t="str">
-        <v>Groomed</v>
+      <c r="D104" s="15" t="str">
+        <v>Dev - WIP</v>
       </c>
       <c r="E104" s="6" t="str">
         <v/>
@@ -4555,7 +4555,7 @@
       <c r="C105" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D105" s="5" t="str">
+      <c r="D105" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E105" s="6" t="str">
@@ -4590,7 +4590,7 @@
       <c r="C106" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D106" s="5" t="str">
+      <c r="D106" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E106" s="6" t="str">
@@ -4625,7 +4625,7 @@
       <c r="C107" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D107" s="11" t="str">
+      <c r="D107" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E107" s="6" t="str">
@@ -4660,8 +4660,8 @@
       <c r="C108" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D108" s="16" t="str">
-        <v>Groomed</v>
+      <c r="D108" s="15" t="str">
+        <v>Dev - WIP</v>
       </c>
       <c r="E108" s="6" t="str">
         <v/>
@@ -4695,8 +4695,8 @@
       <c r="C109" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D109" s="16" t="str">
-        <v>Groomed</v>
+      <c r="D109" s="15" t="str">
+        <v>Dev - WIP</v>
       </c>
       <c r="E109" s="6" t="str">
         <v/>
@@ -4730,8 +4730,8 @@
       <c r="C110" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D110" s="16" t="str">
-        <v>Groomed</v>
+      <c r="D110" s="22" t="str">
+        <v>OnHold</v>
       </c>
       <c r="E110" s="6" t="str">
         <v/>
@@ -4765,7 +4765,7 @@
       <c r="C111" s="6" t="str">
         <v>Richard Whitehouse, Inbal Escholi</v>
       </c>
-      <c r="D111" s="16" t="str">
+      <c r="D111" s="14" t="str">
         <v>Groomed</v>
       </c>
       <c r="E111" s="6" t="str">
@@ -4800,7 +4800,7 @@
       <c r="C112" s="6" t="str">
         <v>Richard Whitehouse</v>
       </c>
-      <c r="D112" s="11" t="str">
+      <c r="D112" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E112" s="6" t="str">
@@ -4835,7 +4835,7 @@
       <c r="C113" s="6" t="str">
         <v>Richard Whitehouse</v>
       </c>
-      <c r="D113" s="17" t="str">
+      <c r="D113" s="18" t="str">
         <v>futureVersion</v>
       </c>
       <c r="E113" s="6" t="str">
@@ -4867,7 +4867,7 @@
       <c r="B114" t="str">
         <v/>
       </c>
-      <c r="C114" s="5" t="str">
+      <c r="C114" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D114" t="str">
@@ -4970,7 +4970,7 @@
       <c r="C116" t="str">
         <v/>
       </c>
-      <c r="D116" s="5" t="str">
+      <c r="D116" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E116" s="6" t="str">
@@ -5005,7 +5005,7 @@
       <c r="C117" t="str">
         <v/>
       </c>
-      <c r="D117" s="5" t="str">
+      <c r="D117" s="15" t="str">
         <v>Dev - WIP</v>
       </c>
       <c r="E117" s="6" t="str">
@@ -5037,7 +5037,7 @@
       <c r="B118" t="str">
         <v/>
       </c>
-      <c r="C118" s="18" t="str">
+      <c r="C118" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="D118" s="6" t="str">
@@ -5102,7 +5102,7 @@
       <c r="B119" t="str">
         <v/>
       </c>
-      <c r="C119" s="17" t="str">
+      <c r="C119" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D119" t="str">
@@ -5205,7 +5205,7 @@
       <c r="C121" t="str">
         <v/>
       </c>
-      <c r="D121" s="14" t="str">
+      <c r="D121" s="13" t="str">
         <v>Handle by other team</v>
       </c>
       <c r="E121" s="6" t="str">
@@ -5240,7 +5240,7 @@
       <c r="C122" t="str">
         <v/>
       </c>
-      <c r="D122" s="14" t="str">
+      <c r="D122" s="13" t="str">
         <v>Handle by other team</v>
       </c>
       <c r="E122" s="6" t="str">
@@ -5275,7 +5275,7 @@
       <c r="C123" t="str">
         <v/>
       </c>
-      <c r="D123" s="19" t="str">
+      <c r="D123" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E123" s="6" t="str">
@@ -5302,12 +5302,12 @@
     </row>
     <row r="124" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="str">
-        <v>Crypto staking</v>
+        <v>Crypto staking - toggles</v>
       </c>
       <c r="B124" t="str">
         <v/>
       </c>
-      <c r="C124" s="14" t="str">
+      <c r="C124" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D124" t="str">
@@ -5323,7 +5323,7 @@
         <v>46141</v>
       </c>
       <c r="H124" s="6" t="str">
-        <v>V2(11.5)</v>
+        <v>V4(8.6)</v>
       </c>
       <c r="I124" t="str">
         <v/>
@@ -5372,7 +5372,7 @@
       <c r="B125" t="str">
         <v/>
       </c>
-      <c r="C125" s="11" t="str">
+      <c r="C125" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D125" t="str">
@@ -5475,7 +5475,7 @@
       <c r="C127" s="6" t="str">
         <v>Hagit Zamir</v>
       </c>
-      <c r="D127" s="11" t="str">
+      <c r="D127" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E127" s="6" t="str">
@@ -5510,7 +5510,7 @@
       <c r="C128" t="str">
         <v/>
       </c>
-      <c r="D128" s="11" t="str">
+      <c r="D128" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E128" s="6" t="str">
@@ -5545,7 +5545,7 @@
       <c r="C129" t="str">
         <v/>
       </c>
-      <c r="D129" s="14" t="str">
+      <c r="D129" s="13" t="str">
         <v>Handle by other team</v>
       </c>
       <c r="E129" s="6" t="str">
@@ -5580,7 +5580,7 @@
       <c r="C130" t="str">
         <v/>
       </c>
-      <c r="D130" s="14" t="str">
+      <c r="D130" s="13" t="str">
         <v>Handle by other team</v>
       </c>
       <c r="E130" s="6" t="str">
@@ -5615,7 +5615,7 @@
       <c r="C131" t="str">
         <v/>
       </c>
-      <c r="D131" s="14" t="str">
+      <c r="D131" s="13" t="str">
         <v>Handle by other team</v>
       </c>
       <c r="E131" s="6" t="str">
@@ -5650,7 +5650,7 @@
       <c r="C132" s="6" t="str">
         <v>Eyal Boas</v>
       </c>
-      <c r="D132" s="19" t="str">
+      <c r="D132" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E132" s="6" t="str">
@@ -5685,7 +5685,7 @@
       <c r="C133" t="str">
         <v/>
       </c>
-      <c r="D133" s="19" t="str">
+      <c r="D133" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E133" s="6" t="str">
@@ -5720,7 +5720,7 @@
       <c r="C134" s="6" t="str">
         <v>Eyal Boas</v>
       </c>
-      <c r="D134" s="19" t="str">
+      <c r="D134" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E134" s="6" t="str">
@@ -5755,7 +5755,7 @@
       <c r="C135" t="str">
         <v/>
       </c>
-      <c r="D135" s="19" t="str">
+      <c r="D135" s="20" t="str">
         <v>Cancelled</v>
       </c>
       <c r="E135" s="6" t="str">
@@ -5787,7 +5787,7 @@
       <c r="B136" t="str">
         <v/>
       </c>
-      <c r="C136" s="15" t="str">
+      <c r="C136" s="16" t="str">
         <v>Grooming</v>
       </c>
       <c r="D136" t="str">
@@ -5890,7 +5890,7 @@
       <c r="C138" t="str">
         <v/>
       </c>
-      <c r="D138" s="20" t="str">
+      <c r="D138" s="17" t="str">
         <v>Grooming</v>
       </c>
       <c r="E138" s="6" t="str">
@@ -5922,7 +5922,7 @@
       <c r="B139" t="str">
         <v/>
       </c>
-      <c r="C139" s="14" t="str">
+      <c r="C139" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D139" s="6" t="str">
@@ -5987,7 +5987,7 @@
       <c r="B140" t="str">
         <v/>
       </c>
-      <c r="C140" s="14" t="str">
+      <c r="C140" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D140" t="str">
@@ -6002,8 +6002,8 @@
       <c r="G140" t="str">
         <v/>
       </c>
-      <c r="H140" t="str">
-        <v/>
+      <c r="H140" s="6" t="str">
+        <v>V3(25.5)</v>
       </c>
       <c r="I140" t="str">
         <v/>
@@ -6052,8 +6052,8 @@
       <c r="B141" t="str">
         <v/>
       </c>
-      <c r="C141" s="5" t="str">
-        <v>FE DEV WIP</v>
+      <c r="C141" s="21" t="str">
+        <v>Cancelled</v>
       </c>
       <c r="D141" t="str">
         <v/>
@@ -6126,10 +6126,10 @@
       <c r="E142" t="str">
         <v/>
       </c>
-      <c r="F142" s="22">
+      <c r="F142" s="23">
         <v>46061</v>
       </c>
-      <c r="G142" s="22">
+      <c r="G142" s="23">
         <v>46160</v>
       </c>
       <c r="H142" t="str">
@@ -6147,7 +6147,7 @@
       <c r="L142" t="str">
         <v/>
       </c>
-      <c r="M142" s="23">
+      <c r="M142" s="24">
         <v>32</v>
       </c>
       <c r="N142" t="str">
@@ -6159,25 +6159,25 @@
       <c r="P142" t="str">
         <v/>
       </c>
-      <c r="Q142" s="24" t="str">
+      <c r="Q142" s="25" t="str">
         <v>2026-02-02 to 2026-04-15</v>
       </c>
       <c r="R142" t="str">
         <v/>
       </c>
-      <c r="S142" s="25" t="str">
-        <v/>
-      </c>
-      <c r="T142" s="22">
+      <c r="S142" s="26" t="str">
+        <v/>
+      </c>
+      <c r="T142" s="23">
         <v>46058</v>
       </c>
-      <c r="U142" s="22">
+      <c r="U142" s="23">
         <v>46114</v>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="144" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A144" s="26" t="str">
+      <c r="A144" s="27" t="str">
         <v>In Focus</v>
       </c>
     </row>
@@ -6253,7 +6253,7 @@
       <c r="B146" t="str">
         <v/>
       </c>
-      <c r="C146" s="11" t="str">
+      <c r="C146" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D146" t="str">
@@ -6318,7 +6318,7 @@
       <c r="B147" t="str">
         <v/>
       </c>
-      <c r="C147" s="14" t="str">
+      <c r="C147" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D147" t="str">
@@ -6383,7 +6383,7 @@
       <c r="B148" t="str">
         <v/>
       </c>
-      <c r="C148" s="14" t="str">
+      <c r="C148" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D148" t="str">
@@ -6448,7 +6448,7 @@
       <c r="B149" t="str">
         <v/>
       </c>
-      <c r="C149" s="27" t="str">
+      <c r="C149" s="28" t="str">
         <v>Risk</v>
       </c>
       <c r="D149" t="str">
@@ -6513,7 +6513,7 @@
       <c r="B150" t="str">
         <v/>
       </c>
-      <c r="C150" s="11" t="str">
+      <c r="C150" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D150" t="str">
@@ -6578,7 +6578,7 @@
       <c r="B151" t="str">
         <v/>
       </c>
-      <c r="C151" s="11" t="str">
+      <c r="C151" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D151" t="str">
@@ -6643,7 +6643,7 @@
       <c r="B152" t="str">
         <v/>
       </c>
-      <c r="C152" s="11" t="str">
+      <c r="C152" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D152" t="str">
@@ -6708,7 +6708,7 @@
       <c r="B153" t="str">
         <v/>
       </c>
-      <c r="C153" s="11" t="str">
+      <c r="C153" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D153" t="str">
@@ -6773,7 +6773,7 @@
       <c r="B154" t="str">
         <v/>
       </c>
-      <c r="C154" s="11" t="str">
+      <c r="C154" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D154" t="str">
@@ -6838,7 +6838,7 @@
       <c r="B155" t="str">
         <v/>
       </c>
-      <c r="C155" s="11" t="str">
+      <c r="C155" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D155" t="str">
@@ -6903,7 +6903,7 @@
       <c r="B156" t="str">
         <v/>
       </c>
-      <c r="C156" s="11" t="str">
+      <c r="C156" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D156" t="str">
@@ -6968,7 +6968,7 @@
       <c r="B157" t="str">
         <v/>
       </c>
-      <c r="C157" s="11" t="str">
+      <c r="C157" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D157" t="str">
@@ -7033,7 +7033,7 @@
       <c r="B158" t="str">
         <v/>
       </c>
-      <c r="C158" s="11" t="str">
+      <c r="C158" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D158" t="str">
@@ -7098,7 +7098,7 @@
       <c r="B159" t="str">
         <v/>
       </c>
-      <c r="C159" s="11" t="str">
+      <c r="C159" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D159" t="str">
@@ -7163,7 +7163,7 @@
       <c r="B160" t="str">
         <v/>
       </c>
-      <c r="C160" s="11" t="str">
+      <c r="C160" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D160" s="6" t="str">
@@ -7228,7 +7228,7 @@
       <c r="B161" t="str">
         <v/>
       </c>
-      <c r="C161" s="11" t="str">
+      <c r="C161" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D161" t="str">
@@ -7293,7 +7293,7 @@
       <c r="B162" t="str">
         <v/>
       </c>
-      <c r="C162" s="11" t="str">
+      <c r="C162" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D162" t="str">
@@ -7358,7 +7358,7 @@
       <c r="B163" t="str">
         <v/>
       </c>
-      <c r="C163" s="11" t="str">
+      <c r="C163" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D163" t="str">
@@ -7423,7 +7423,7 @@
       <c r="B164" t="str">
         <v/>
       </c>
-      <c r="C164" s="11" t="str">
+      <c r="C164" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D164" t="str">
@@ -7488,7 +7488,7 @@
       <c r="B165" t="str">
         <v/>
       </c>
-      <c r="C165" s="11" t="str">
+      <c r="C165" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D165" t="str">
@@ -7553,7 +7553,7 @@
       <c r="B166" t="str">
         <v/>
       </c>
-      <c r="C166" s="11" t="str">
+      <c r="C166" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D166" t="str">
@@ -7618,7 +7618,7 @@
       <c r="B167" t="str">
         <v/>
       </c>
-      <c r="C167" s="11" t="str">
+      <c r="C167" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D167" t="str">
@@ -7692,10 +7692,10 @@
       <c r="E168" t="str">
         <v/>
       </c>
-      <c r="F168" s="22">
+      <c r="F168" s="23">
         <v>46054</v>
       </c>
-      <c r="G168" s="22">
+      <c r="G168" s="23">
         <v>46118</v>
       </c>
       <c r="H168" t="str">
@@ -7713,7 +7713,7 @@
       <c r="L168" t="str">
         <v/>
       </c>
-      <c r="M168" s="23">
+      <c r="M168" s="24">
         <v>0</v>
       </c>
       <c r="N168" t="str">
@@ -7725,25 +7725,25 @@
       <c r="P168" t="str">
         <v/>
       </c>
-      <c r="Q168" s="25" t="str">
+      <c r="Q168" s="26" t="str">
         <v/>
       </c>
       <c r="R168" t="str">
         <v/>
       </c>
-      <c r="S168" s="25" t="str">
-        <v/>
-      </c>
-      <c r="T168" s="25" t="str">
-        <v/>
-      </c>
-      <c r="U168" s="25" t="str">
+      <c r="S168" s="26" t="str">
+        <v/>
+      </c>
+      <c r="T168" s="26" t="str">
+        <v/>
+      </c>
+      <c r="U168" s="26" t="str">
         <v/>
       </c>
     </row>
     <row r="169" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="170" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" s="28" t="str">
+      <c r="A170" s="29" t="str">
         <v>MVP - API /BFF project</v>
       </c>
     </row>
@@ -7819,7 +7819,7 @@
       <c r="B172" t="str">
         <v/>
       </c>
-      <c r="C172" s="11" t="str">
+      <c r="C172" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D172" s="6" t="str">
@@ -7922,7 +7922,7 @@
       <c r="C174" t="str">
         <v/>
       </c>
-      <c r="D174" s="11" t="str">
+      <c r="D174" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E174" s="6" t="str">
@@ -7957,7 +7957,7 @@
       <c r="C175" t="str">
         <v/>
       </c>
-      <c r="D175" s="11" t="str">
+      <c r="D175" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E175" s="6" t="str">
@@ -7992,7 +7992,7 @@
       <c r="C176" s="6" t="str">
         <v>Hagit Zamir</v>
       </c>
-      <c r="D176" s="11" t="str">
+      <c r="D176" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E176" s="6" t="str">
@@ -8027,7 +8027,7 @@
       <c r="C177" t="str">
         <v/>
       </c>
-      <c r="D177" s="11" t="str">
+      <c r="D177" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E177" s="6" t="str">
@@ -8062,7 +8062,7 @@
       <c r="C178" t="str">
         <v/>
       </c>
-      <c r="D178" s="11" t="str">
+      <c r="D178" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E178" s="6" t="str">
@@ -8097,7 +8097,7 @@
       <c r="C179" t="str">
         <v/>
       </c>
-      <c r="D179" s="11" t="str">
+      <c r="D179" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E179" s="6" t="str">
@@ -8132,7 +8132,7 @@
       <c r="C180" t="str">
         <v/>
       </c>
-      <c r="D180" s="11" t="str">
+      <c r="D180" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E180" s="6" t="str">
@@ -8164,7 +8164,7 @@
       <c r="B181" t="str">
         <v/>
       </c>
-      <c r="C181" s="11" t="str">
+      <c r="C181" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D181" s="6" t="str">
@@ -8229,7 +8229,7 @@
       <c r="B182" t="str">
         <v/>
       </c>
-      <c r="C182" s="11" t="str">
+      <c r="C182" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D182" s="6" t="str">
@@ -8332,7 +8332,7 @@
       <c r="C184" t="str">
         <v/>
       </c>
-      <c r="D184" s="11" t="str">
+      <c r="D184" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E184" s="6" t="str">
@@ -8367,7 +8367,7 @@
       <c r="C185" t="str">
         <v/>
       </c>
-      <c r="D185" s="11" t="str">
+      <c r="D185" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E185" s="6" t="str">
@@ -8402,7 +8402,7 @@
       <c r="C186" t="str">
         <v/>
       </c>
-      <c r="D186" s="11" t="str">
+      <c r="D186" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E186" s="6" t="str">
@@ -8437,7 +8437,7 @@
       <c r="C187" t="str">
         <v/>
       </c>
-      <c r="D187" s="11" t="str">
+      <c r="D187" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E187" s="6" t="str">
@@ -8472,7 +8472,7 @@
       <c r="C188" t="str">
         <v/>
       </c>
-      <c r="D188" s="11" t="str">
+      <c r="D188" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E188" s="6" t="str">
@@ -8507,7 +8507,7 @@
       <c r="C189" t="str">
         <v/>
       </c>
-      <c r="D189" s="11" t="str">
+      <c r="D189" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="E189" s="6" t="str">
@@ -8539,7 +8539,7 @@
       <c r="B190" t="str">
         <v/>
       </c>
-      <c r="C190" s="11" t="str">
+      <c r="C190" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D190" t="str">
@@ -8604,7 +8604,7 @@
       <c r="B191" t="str">
         <v/>
       </c>
-      <c r="C191" s="18" t="str">
+      <c r="C191" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="D191" t="str">
@@ -8669,7 +8669,7 @@
       <c r="B192" t="str">
         <v/>
       </c>
-      <c r="C192" s="11" t="str">
+      <c r="C192" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D192" t="str">
@@ -8734,7 +8734,7 @@
       <c r="B193" t="str">
         <v/>
       </c>
-      <c r="C193" s="18" t="str">
+      <c r="C193" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="D193" s="6" t="str">
@@ -8799,7 +8799,7 @@
       <c r="B194" t="str">
         <v/>
       </c>
-      <c r="C194" s="12" t="str">
+      <c r="C194" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="D194" s="6" t="str">
@@ -8902,7 +8902,7 @@
       <c r="C196" t="str">
         <v/>
       </c>
-      <c r="D196" s="12" t="str">
+      <c r="D196" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="E196" s="6" t="str">
@@ -8934,7 +8934,7 @@
       <c r="B197" t="str">
         <v/>
       </c>
-      <c r="C197" s="12" t="str">
+      <c r="C197" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="D197" s="6" t="str">
@@ -8999,7 +8999,7 @@
       <c r="B198" t="str">
         <v/>
       </c>
-      <c r="C198" s="12" t="str">
+      <c r="C198" s="11" t="str">
         <v>Stuck</v>
       </c>
       <c r="D198" s="6" t="str">
@@ -9064,7 +9064,7 @@
       <c r="B199" t="str">
         <v/>
       </c>
-      <c r="C199" s="18" t="str">
+      <c r="C199" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="D199" s="6" t="str">
@@ -9129,7 +9129,7 @@
       <c r="B200" t="str">
         <v/>
       </c>
-      <c r="C200" s="18" t="str">
+      <c r="C200" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="D200" s="6" t="str">
@@ -9194,7 +9194,7 @@
       <c r="B201" t="str">
         <v/>
       </c>
-      <c r="C201" s="14" t="str">
+      <c r="C201" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D201" t="str">
@@ -9259,7 +9259,7 @@
       <c r="B202" t="str">
         <v/>
       </c>
-      <c r="C202" s="14" t="str">
+      <c r="C202" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D202" t="str">
@@ -9454,7 +9454,7 @@
       <c r="B205" t="str">
         <v/>
       </c>
-      <c r="C205" s="17" t="str">
+      <c r="C205" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D205" s="6" t="str">
@@ -9528,10 +9528,10 @@
       <c r="E206" t="str">
         <v/>
       </c>
-      <c r="F206" s="22">
+      <c r="F206" s="23">
         <v>46036</v>
       </c>
-      <c r="G206" s="22">
+      <c r="G206" s="23">
         <v>46134</v>
       </c>
       <c r="H206" t="str">
@@ -9549,7 +9549,7 @@
       <c r="L206" t="str">
         <v/>
       </c>
-      <c r="M206" s="23">
+      <c r="M206" s="24">
         <v>9</v>
       </c>
       <c r="N206" t="str">
@@ -9561,25 +9561,25 @@
       <c r="P206" t="str">
         <v/>
       </c>
-      <c r="Q206" s="25" t="str">
+      <c r="Q206" s="26" t="str">
         <v/>
       </c>
       <c r="R206" t="str">
         <v/>
       </c>
-      <c r="S206" s="25" t="str">
-        <v/>
-      </c>
-      <c r="T206" s="25" t="str">
-        <v/>
-      </c>
-      <c r="U206" s="25" t="str">
+      <c r="S206" s="26" t="str">
+        <v/>
+      </c>
+      <c r="T206" s="26" t="str">
+        <v/>
+      </c>
+      <c r="U206" s="26" t="str">
         <v/>
       </c>
     </row>
     <row r="207" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="208" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A208" s="29" t="str">
+      <c r="A208" s="30" t="str">
         <v>Not in Money scope/Future versions</v>
       </c>
     </row>
@@ -9655,7 +9655,7 @@
       <c r="B210" t="str">
         <v/>
       </c>
-      <c r="C210" s="17" t="str">
+      <c r="C210" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D210" s="6" t="str">
@@ -9720,7 +9720,7 @@
       <c r="B211" t="str">
         <v/>
       </c>
-      <c r="C211" s="17" t="str">
+      <c r="C211" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D211" s="6" t="str">
@@ -9785,7 +9785,7 @@
       <c r="B212" t="str">
         <v/>
       </c>
-      <c r="C212" s="17" t="str">
+      <c r="C212" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D212" s="6" t="str">
@@ -9850,7 +9850,7 @@
       <c r="B213" t="str">
         <v/>
       </c>
-      <c r="C213" s="17" t="str">
+      <c r="C213" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D213" s="6" t="str">
@@ -9915,7 +9915,7 @@
       <c r="B214" t="str">
         <v/>
       </c>
-      <c r="C214" s="17" t="str">
+      <c r="C214" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D214" s="6" t="str">
@@ -9981,7 +9981,7 @@
       <c r="B215" t="str">
         <v/>
       </c>
-      <c r="C215" s="17" t="str">
+      <c r="C215" s="18" t="str">
         <v>Managed by other team</v>
       </c>
       <c r="D215" s="6" t="str">
@@ -10084,7 +10084,7 @@
       <c r="C217" t="str">
         <v/>
       </c>
-      <c r="D217" s="18" t="str">
+      <c r="D217" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="E217" s="6" t="str">
@@ -10119,7 +10119,7 @@
       <c r="C218" t="str">
         <v/>
       </c>
-      <c r="D218" s="18" t="str">
+      <c r="D218" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="E218" s="6" t="str">
@@ -10151,7 +10151,7 @@
       <c r="B219" t="str">
         <v/>
       </c>
-      <c r="C219" s="30" t="str">
+      <c r="C219" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D219" s="6" t="str">
@@ -10216,7 +10216,7 @@
       <c r="B220" t="str">
         <v/>
       </c>
-      <c r="C220" s="30" t="str">
+      <c r="C220" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D220" s="6" t="str">
@@ -10281,7 +10281,7 @@
       <c r="B221" t="str">
         <v/>
       </c>
-      <c r="C221" s="30" t="str">
+      <c r="C221" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D221" t="str">
@@ -10384,7 +10384,7 @@
       <c r="C223" t="str">
         <v/>
       </c>
-      <c r="D223" s="18" t="str">
+      <c r="D223" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="E223" s="6" t="str">
@@ -10419,7 +10419,7 @@
       <c r="C224" t="str">
         <v/>
       </c>
-      <c r="D224" s="18" t="str">
+      <c r="D224" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="E224" s="6" t="str">
@@ -10451,7 +10451,7 @@
       <c r="B225" t="str">
         <v/>
       </c>
-      <c r="C225" s="30" t="str">
+      <c r="C225" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D225" s="6" t="str">
@@ -10516,7 +10516,7 @@
       <c r="B226" t="str">
         <v/>
       </c>
-      <c r="C226" s="30" t="str">
+      <c r="C226" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D226" s="6" t="str">
@@ -10581,7 +10581,7 @@
       <c r="B227" t="str">
         <v/>
       </c>
-      <c r="C227" s="30" t="str">
+      <c r="C227" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D227" t="str">
@@ -10646,7 +10646,7 @@
       <c r="B228" t="str">
         <v/>
       </c>
-      <c r="C228" s="30" t="str">
+      <c r="C228" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D228" t="str">
@@ -10711,7 +10711,7 @@
       <c r="B229" t="str">
         <v/>
       </c>
-      <c r="C229" s="30" t="str">
+      <c r="C229" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D229" s="6" t="str">
@@ -11036,7 +11036,7 @@
       <c r="B234" t="str">
         <v/>
       </c>
-      <c r="C234" s="30" t="str">
+      <c r="C234" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D234" t="str">
@@ -11101,7 +11101,7 @@
       <c r="B235" t="str">
         <v/>
       </c>
-      <c r="C235" s="30" t="str">
+      <c r="C235" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D235" s="6" t="str">
@@ -11175,10 +11175,10 @@
       <c r="E236" t="str">
         <v/>
       </c>
-      <c r="F236" s="22">
+      <c r="F236" s="23">
         <v>46061</v>
       </c>
-      <c r="G236" s="22">
+      <c r="G236" s="23">
         <v>46134</v>
       </c>
       <c r="H236" t="str">
@@ -11196,7 +11196,7 @@
       <c r="L236" t="str">
         <v/>
       </c>
-      <c r="M236" s="23">
+      <c r="M236" s="24">
         <v>1298</v>
       </c>
       <c r="N236" t="str">
@@ -11208,19 +11208,19 @@
       <c r="P236" t="str">
         <v/>
       </c>
-      <c r="Q236" s="24" t="str">
+      <c r="Q236" s="25" t="str">
         <v>2026-03-02 to 2026-03-23</v>
       </c>
       <c r="R236" t="str">
         <v/>
       </c>
-      <c r="S236" s="25" t="str">
-        <v/>
-      </c>
-      <c r="T236" s="22">
+      <c r="S236" s="26" t="str">
+        <v/>
+      </c>
+      <c r="T236" s="23">
         <v>46104</v>
       </c>
-      <c r="U236" s="22">
+      <c r="U236" s="23">
         <v>46104</v>
       </c>
     </row>
@@ -11302,7 +11302,7 @@
       <c r="B240" t="str">
         <v/>
       </c>
-      <c r="C240" s="11" t="str">
+      <c r="C240" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D240" t="str">
@@ -11367,7 +11367,7 @@
       <c r="B241" t="str">
         <v/>
       </c>
-      <c r="C241" s="5" t="str">
+      <c r="C241" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D241" t="str">
@@ -11432,7 +11432,7 @@
       <c r="B242" t="str">
         <v/>
       </c>
-      <c r="C242" s="5" t="str">
+      <c r="C242" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D242" t="str">
@@ -11497,7 +11497,7 @@
       <c r="B243" t="str">
         <v/>
       </c>
-      <c r="C243" s="18" t="str">
+      <c r="C243" s="19" t="str">
         <v>Not Started</v>
       </c>
       <c r="D243" t="str">
@@ -11562,7 +11562,7 @@
       <c r="B244" t="str">
         <v/>
       </c>
-      <c r="C244" s="16" t="str">
+      <c r="C244" s="14" t="str">
         <v>Deployment</v>
       </c>
       <c r="D244" t="str">
@@ -11627,7 +11627,7 @@
       <c r="B245" t="str">
         <v/>
       </c>
-      <c r="C245" s="5" t="str">
+      <c r="C245" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D245" t="str">
@@ -11692,7 +11692,7 @@
       <c r="B246" t="str">
         <v/>
       </c>
-      <c r="C246" s="5" t="str">
+      <c r="C246" s="15" t="str">
         <v>FE DEV WIP</v>
       </c>
       <c r="D246" t="str">
@@ -11757,7 +11757,7 @@
       <c r="B247" t="str">
         <v/>
       </c>
-      <c r="C247" s="14" t="str">
+      <c r="C247" s="13" t="str">
         <v>Discovery</v>
       </c>
       <c r="D247" t="str">
@@ -11831,10 +11831,10 @@
       <c r="E248" t="str">
         <v/>
       </c>
-      <c r="F248" s="22">
+      <c r="F248" s="23">
         <v>46048</v>
       </c>
-      <c r="G248" s="22">
+      <c r="G248" s="23">
         <v>46145</v>
       </c>
       <c r="H248" t="str">
@@ -11852,7 +11852,7 @@
       <c r="L248" t="str">
         <v/>
       </c>
-      <c r="M248" s="23">
+      <c r="M248" s="24">
         <v>0</v>
       </c>
       <c r="N248" t="str">
@@ -11864,25 +11864,25 @@
       <c r="P248" t="str">
         <v/>
       </c>
-      <c r="Q248" s="25" t="str">
+      <c r="Q248" s="26" t="str">
         <v/>
       </c>
       <c r="R248" t="str">
         <v/>
       </c>
-      <c r="S248" s="25" t="str">
-        <v/>
-      </c>
-      <c r="T248" s="25" t="str">
-        <v/>
-      </c>
-      <c r="U248" s="25" t="str">
+      <c r="S248" s="26" t="str">
+        <v/>
+      </c>
+      <c r="T248" s="26" t="str">
+        <v/>
+      </c>
+      <c r="U248" s="26" t="str">
         <v/>
       </c>
     </row>
     <row r="249" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="250" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A250" s="26" t="str">
+      <c r="A250" s="27" t="str">
         <v>Dependencies</v>
       </c>
     </row>
@@ -11958,7 +11958,7 @@
       <c r="B252" t="str">
         <v/>
       </c>
-      <c r="C252" s="11" t="str">
+      <c r="C252" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D252" t="str">
@@ -12088,7 +12088,7 @@
       <c r="B254" t="str">
         <v/>
       </c>
-      <c r="C254" s="11" t="str">
+      <c r="C254" s="12" t="str">
         <v>Done</v>
       </c>
       <c r="D254" t="str">
@@ -12162,10 +12162,10 @@
       <c r="E255" t="str">
         <v/>
       </c>
-      <c r="F255" s="25" t="str">
-        <v/>
-      </c>
-      <c r="G255" s="25" t="str">
+      <c r="F255" s="26" t="str">
+        <v/>
+      </c>
+      <c r="G255" s="26" t="str">
         <v/>
       </c>
       <c r="H255" t="str">
@@ -12183,7 +12183,7 @@
       <c r="L255" t="str">
         <v/>
       </c>
-      <c r="M255" s="23">
+      <c r="M255" s="24">
         <v>0</v>
       </c>
       <c r="N255" t="str">
@@ -12195,19 +12195,19 @@
       <c r="P255" t="str">
         <v/>
       </c>
-      <c r="Q255" s="25" t="str">
+      <c r="Q255" s="26" t="str">
         <v/>
       </c>
       <c r="R255" t="str">
         <v/>
       </c>
-      <c r="S255" s="25" t="str">
-        <v/>
-      </c>
-      <c r="T255" s="25" t="str">
-        <v/>
-      </c>
-      <c r="U255" s="25" t="str">
+      <c r="S255" s="26" t="str">
+        <v/>
+      </c>
+      <c r="T255" s="26" t="str">
+        <v/>
+      </c>
+      <c r="U255" s="26" t="str">
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh roadmap from Monday Excel export (eToro_Plus_Money_1779269565)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/board-export.xlsx
+++ b/data/board-export.xlsx
@@ -148,17 +148,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF5AC4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF757575"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF66CCFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF5AC4"/>
       </patternFill>
     </fill>
   </fills>
@@ -240,6 +240,9 @@
     <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -253,7 +256,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -261,9 +264,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4180,8 +4180,8 @@
       <c r="B95" t="str">
         <v/>
       </c>
-      <c r="C95" s="12" t="str">
-        <v>Stuck</v>
+      <c r="C95" s="22" t="str">
+        <v>Future Version</v>
       </c>
       <c r="D95" s="6" t="str">
         <v>withdrawWizard</v>
@@ -5410,7 +5410,7 @@
       <c r="B125" t="str">
         <v/>
       </c>
-      <c r="C125" s="22" t="str">
+      <c r="C125" s="23" t="str">
         <v>Groomed</v>
       </c>
       <c r="D125" t="str">
@@ -5950,8 +5950,8 @@
       <c r="G134" t="str">
         <v/>
       </c>
-      <c r="H134" t="str">
-        <v/>
+      <c r="H134" s="6" t="str">
+        <v>V3(25.5)</v>
       </c>
       <c r="I134" t="str">
         <v/>
@@ -6009,10 +6009,10 @@
       <c r="E135" t="str">
         <v/>
       </c>
-      <c r="F135" s="23">
+      <c r="F135" s="24">
         <v>46061</v>
       </c>
-      <c r="G135" s="23">
+      <c r="G135" s="24">
         <v>46160</v>
       </c>
       <c r="H135" t="str">
@@ -6030,7 +6030,7 @@
       <c r="L135" t="str">
         <v/>
       </c>
-      <c r="M135" s="24">
+      <c r="M135" s="25">
         <v>30</v>
       </c>
       <c r="N135" t="str">
@@ -6042,25 +6042,25 @@
       <c r="P135" t="str">
         <v/>
       </c>
-      <c r="Q135" s="25" t="str">
+      <c r="Q135" s="26" t="str">
         <v>2026-02-02 to 2026-04-15</v>
       </c>
       <c r="R135" t="str">
         <v/>
       </c>
-      <c r="S135" s="26" t="str">
-        <v/>
-      </c>
-      <c r="T135" s="23">
+      <c r="S135" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T135" s="24">
         <v>46058</v>
       </c>
-      <c r="U135" s="23">
+      <c r="U135" s="24">
         <v>46114</v>
       </c>
     </row>
     <row r="136" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="137" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A137" s="27" t="str">
+      <c r="A137" s="28" t="str">
         <v>In Focus</v>
       </c>
     </row>
@@ -6331,7 +6331,7 @@
       <c r="B142" t="str">
         <v/>
       </c>
-      <c r="C142" s="28" t="str">
+      <c r="C142" s="29" t="str">
         <v>Risk</v>
       </c>
       <c r="D142" t="str">
@@ -7640,10 +7640,10 @@
       <c r="E162" t="str">
         <v/>
       </c>
-      <c r="F162" s="23">
+      <c r="F162" s="24">
         <v>46054</v>
       </c>
-      <c r="G162" s="23">
+      <c r="G162" s="24">
         <v>46118</v>
       </c>
       <c r="H162" t="str">
@@ -7661,7 +7661,7 @@
       <c r="L162" t="str">
         <v/>
       </c>
-      <c r="M162" s="24">
+      <c r="M162" s="25">
         <v>0</v>
       </c>
       <c r="N162" t="str">
@@ -7673,25 +7673,25 @@
       <c r="P162" t="str">
         <v/>
       </c>
-      <c r="Q162" s="26" t="str">
+      <c r="Q162" s="27" t="str">
         <v/>
       </c>
       <c r="R162" t="str">
         <v/>
       </c>
-      <c r="S162" s="26" t="str">
-        <v/>
-      </c>
-      <c r="T162" s="26" t="str">
-        <v/>
-      </c>
-      <c r="U162" s="26" t="str">
+      <c r="S162" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T162" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U162" s="27" t="str">
         <v/>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="164" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" s="29" t="str">
+      <c r="A164" s="30" t="str">
         <v>MVP - API /BFF project</v>
       </c>
     </row>
@@ -9891,10 +9891,10 @@
       <c r="E211" t="str">
         <v/>
       </c>
-      <c r="F211" s="23">
+      <c r="F211" s="24">
         <v>46036</v>
       </c>
-      <c r="G211" s="23">
+      <c r="G211" s="24">
         <v>46134</v>
       </c>
       <c r="H211" t="str">
@@ -9912,7 +9912,7 @@
       <c r="L211" t="str">
         <v/>
       </c>
-      <c r="M211" s="24">
+      <c r="M211" s="25">
         <v>11</v>
       </c>
       <c r="N211" t="str">
@@ -9924,25 +9924,25 @@
       <c r="P211" t="str">
         <v/>
       </c>
-      <c r="Q211" s="26" t="str">
+      <c r="Q211" s="27" t="str">
         <v/>
       </c>
       <c r="R211" t="str">
         <v/>
       </c>
-      <c r="S211" s="26" t="str">
-        <v/>
-      </c>
-      <c r="T211" s="26" t="str">
-        <v/>
-      </c>
-      <c r="U211" s="26" t="str">
+      <c r="S211" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T211" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U211" s="27" t="str">
         <v/>
       </c>
     </row>
     <row r="212" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="213" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A213" s="30" t="str">
+      <c r="A213" s="31" t="str">
         <v>Not in Money scope/Future versions</v>
       </c>
     </row>
@@ -10514,7 +10514,7 @@
       <c r="B224" t="str">
         <v/>
       </c>
-      <c r="C224" s="31" t="str">
+      <c r="C224" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D224" s="6" t="str">
@@ -10579,7 +10579,7 @@
       <c r="B225" t="str">
         <v/>
       </c>
-      <c r="C225" s="31" t="str">
+      <c r="C225" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D225" s="6" t="str">
@@ -10644,7 +10644,7 @@
       <c r="B226" t="str">
         <v/>
       </c>
-      <c r="C226" s="31" t="str">
+      <c r="C226" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D226" t="str">
@@ -10814,7 +10814,7 @@
       <c r="B230" t="str">
         <v/>
       </c>
-      <c r="C230" s="31" t="str">
+      <c r="C230" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D230" s="6" t="str">
@@ -10879,7 +10879,7 @@
       <c r="B231" t="str">
         <v/>
       </c>
-      <c r="C231" s="31" t="str">
+      <c r="C231" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D231" s="6" t="str">
@@ -10944,7 +10944,7 @@
       <c r="B232" t="str">
         <v/>
       </c>
-      <c r="C232" s="31" t="str">
+      <c r="C232" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D232" t="str">
@@ -11009,7 +11009,7 @@
       <c r="B233" t="str">
         <v/>
       </c>
-      <c r="C233" s="31" t="str">
+      <c r="C233" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D233" t="str">
@@ -11074,7 +11074,7 @@
       <c r="B234" t="str">
         <v/>
       </c>
-      <c r="C234" s="31" t="str">
+      <c r="C234" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D234" s="6" t="str">
@@ -11399,7 +11399,7 @@
       <c r="B239" t="str">
         <v/>
       </c>
-      <c r="C239" s="31" t="str">
+      <c r="C239" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D239" t="str">
@@ -11464,7 +11464,7 @@
       <c r="B240" t="str">
         <v/>
       </c>
-      <c r="C240" s="31" t="str">
+      <c r="C240" s="22" t="str">
         <v>Future Version</v>
       </c>
       <c r="D240" s="6" t="str">
@@ -11538,10 +11538,10 @@
       <c r="E241" t="str">
         <v/>
       </c>
-      <c r="F241" s="23">
+      <c r="F241" s="24">
         <v>46061</v>
       </c>
-      <c r="G241" s="23">
+      <c r="G241" s="24">
         <v>46134</v>
       </c>
       <c r="H241" t="str">
@@ -11559,7 +11559,7 @@
       <c r="L241" t="str">
         <v/>
       </c>
-      <c r="M241" s="24">
+      <c r="M241" s="25">
         <v>1298</v>
       </c>
       <c r="N241" t="str">
@@ -11571,19 +11571,19 @@
       <c r="P241" t="str">
         <v/>
       </c>
-      <c r="Q241" s="25" t="str">
+      <c r="Q241" s="26" t="str">
         <v>2026-03-02 to 2026-03-23</v>
       </c>
       <c r="R241" t="str">
         <v/>
       </c>
-      <c r="S241" s="26" t="str">
-        <v/>
-      </c>
-      <c r="T241" s="23">
+      <c r="S241" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T241" s="24">
         <v>46104</v>
       </c>
-      <c r="U241" s="23">
+      <c r="U241" s="24">
         <v>46104</v>
       </c>
     </row>
@@ -12194,10 +12194,10 @@
       <c r="E253" t="str">
         <v/>
       </c>
-      <c r="F253" s="23">
+      <c r="F253" s="24">
         <v>46048</v>
       </c>
-      <c r="G253" s="23">
+      <c r="G253" s="24">
         <v>46145</v>
       </c>
       <c r="H253" t="str">
@@ -12215,7 +12215,7 @@
       <c r="L253" t="str">
         <v/>
       </c>
-      <c r="M253" s="24">
+      <c r="M253" s="25">
         <v>0</v>
       </c>
       <c r="N253" t="str">
@@ -12227,25 +12227,25 @@
       <c r="P253" t="str">
         <v/>
       </c>
-      <c r="Q253" s="26" t="str">
+      <c r="Q253" s="27" t="str">
         <v/>
       </c>
       <c r="R253" t="str">
         <v/>
       </c>
-      <c r="S253" s="26" t="str">
-        <v/>
-      </c>
-      <c r="T253" s="26" t="str">
-        <v/>
-      </c>
-      <c r="U253" s="26" t="str">
+      <c r="S253" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T253" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U253" s="27" t="str">
         <v/>
       </c>
     </row>
     <row r="254" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="255" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A255" s="27" t="str">
+      <c r="A255" s="28" t="str">
         <v>Dependencies</v>
       </c>
     </row>
@@ -12525,10 +12525,10 @@
       <c r="E260" t="str">
         <v/>
       </c>
-      <c r="F260" s="26" t="str">
-        <v/>
-      </c>
-      <c r="G260" s="26" t="str">
+      <c r="F260" s="27" t="str">
+        <v/>
+      </c>
+      <c r="G260" s="27" t="str">
         <v/>
       </c>
       <c r="H260" t="str">
@@ -12546,7 +12546,7 @@
       <c r="L260" t="str">
         <v/>
       </c>
-      <c r="M260" s="24">
+      <c r="M260" s="25">
         <v>0</v>
       </c>
       <c r="N260" t="str">
@@ -12558,19 +12558,19 @@
       <c r="P260" t="str">
         <v/>
       </c>
-      <c r="Q260" s="26" t="str">
+      <c r="Q260" s="27" t="str">
         <v/>
       </c>
       <c r="R260" t="str">
         <v/>
       </c>
-      <c r="S260" s="26" t="str">
-        <v/>
-      </c>
-      <c r="T260" s="26" t="str">
-        <v/>
-      </c>
-      <c r="U260" s="26" t="str">
+      <c r="S260" s="27" t="str">
+        <v/>
+      </c>
+      <c r="T260" s="27" t="str">
+        <v/>
+      </c>
+      <c r="U260" s="27" t="str">
         <v/>
       </c>
     </row>

</xml_diff>